<commit_message>
Update latest results (2026-05-19_19-54-13)
</commit_message>
<xml_diff>
--- a/res/csv/data_by_date.xlsx
+++ b/res/csv/data_by_date.xlsx
@@ -1283,7 +1283,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>over: 1555.52 &gt; 80.0</t>
+          <t>over: 1555.52 &gt; 60.0</t>
         </is>
       </c>
       <c r="O16" t="b">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>over: 2122.60 &gt; 80.0</t>
+          <t>over: 2122.60 &gt; 60.0</t>
         </is>
       </c>
       <c r="O17" t="b">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>over: 78633.94 &gt; 80.0</t>
+          <t>over: 78633.94 &gt; 60.0</t>
         </is>
       </c>
       <c r="O18" t="b">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>over: 8247.89 &gt; 80.0</t>
+          <t>over: 8247.89 &gt; 60.0</t>
         </is>
       </c>
       <c r="O19" t="b">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>over: 31978.97 &gt; 80.0</t>
+          <t>over: 31978.97 &gt; 60.0</t>
         </is>
       </c>
       <c r="O20" t="b">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>over: 4293.41 &gt; 80.0</t>
+          <t>over: 4293.41 &gt; 60.0</t>
         </is>
       </c>
       <c r="O21" t="b">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>over: 1062.17 &gt; 80.0</t>
+          <t>over: 1062.17 &gt; 60.0</t>
         </is>
       </c>
       <c r="O22" t="b">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>over: 3053.87 &gt; 80.0</t>
+          <t>over: 3053.87 &gt; 60.0</t>
         </is>
       </c>
       <c r="O23" t="b">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>over: 23325.19 &gt; 80.0</t>
+          <t>over: 23325.19 &gt; 60.0</t>
         </is>
       </c>
       <c r="O24" t="b">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>over: 4083.92 &gt; 80.0</t>
+          <t>over: 4083.92 &gt; 60.0</t>
         </is>
       </c>
       <c r="O25" t="b">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>over: 3649.45 &gt; 80.0</t>
+          <t>over: 3649.45 &gt; 60.0</t>
         </is>
       </c>
       <c r="O26" t="b">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>over: 2157.59 &gt; 80.0</t>
+          <t>over: 2157.59 &gt; 60.0</t>
         </is>
       </c>
       <c r="O27" t="b">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>over: 64881.05 &gt; 80.0</t>
+          <t>over: 64881.05 &gt; 60.0</t>
         </is>
       </c>
       <c r="O28" t="b">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>over: 3778.30 &gt; 80.0</t>
+          <t>over: 3778.30 &gt; 60.0</t>
         </is>
       </c>
       <c r="O29" t="b">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>over: 5340.69 &gt; 80.0</t>
+          <t>over: 5340.69 &gt; 60.0</t>
         </is>
       </c>
       <c r="O30" t="b">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>over: 17795.66 &gt; 80.0</t>
+          <t>over: 17795.66 &gt; 60.0</t>
         </is>
       </c>
       <c r="O31" t="b">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>over: 18100.32 &gt; 80.0</t>
+          <t>over: 18100.32 &gt; 60.0</t>
         </is>
       </c>
       <c r="O32" t="b">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>over: 3659.56 &gt; 80.0</t>
+          <t>over: 3659.56 &gt; 60.0</t>
         </is>
       </c>
       <c r="O33" t="b">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>over: 8031.53 &gt; 80.0</t>
+          <t>over: 8031.53 &gt; 60.0</t>
         </is>
       </c>
       <c r="O34" t="b">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>over: 16295.70 &gt; 80.0</t>
+          <t>over: 16295.70 &gt; 60.0</t>
         </is>
       </c>
       <c r="O35" t="b">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>over: 2781.36 &gt; 80.0</t>
+          <t>over: 2781.36 &gt; 60.0</t>
         </is>
       </c>
       <c r="O36" t="b">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>over: 2688.22 &gt; 80.0</t>
+          <t>over: 2688.22 &gt; 60.0</t>
         </is>
       </c>
       <c r="O37" t="b">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>over: 8688.93 &gt; 80.0</t>
+          <t>over: 8688.93 &gt; 60.0</t>
         </is>
       </c>
       <c r="O38" t="b">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>over: 46254.71 &gt; 80.0</t>
+          <t>over: 46254.71 &gt; 60.0</t>
         </is>
       </c>
       <c r="O39" t="b">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>over: 1429.78 &gt; 80.0</t>
+          <t>over: 1429.78 &gt; 60.0</t>
         </is>
       </c>
       <c r="O40" t="b">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>over: 5666.98 &gt; 80.0</t>
+          <t>over: 5666.98 &gt; 60.0</t>
         </is>
       </c>
       <c r="O41" t="b">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>over: 5615.99 &gt; 80.0</t>
+          <t>over: 5615.99 &gt; 60.0</t>
         </is>
       </c>
       <c r="O42" t="b">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>over: 7012.52 &gt; 80.0</t>
+          <t>over: 7012.52 &gt; 60.0</t>
         </is>
       </c>
       <c r="O43" t="b">
@@ -4176,7 +4176,7 @@
       <c r="F72" t="n">
         <v>450</v>
       </c>
-      <c r="G72" t="n">
+      <c r="G72" s="2" t="n">
         <v>36.843</v>
       </c>
       <c r="H72" t="n">
@@ -4185,9 +4185,13 @@
       <c r="I72" t="n">
         <v>32.32</v>
       </c>
-      <c r="J72" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.84 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="b">
@@ -4197,8 +4201,8 @@
       <c r="O72" t="b">
         <v>0</v>
       </c>
-      <c r="P72" t="b">
-        <v>0</v>
+      <c r="P72" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4226,7 +4230,7 @@
       <c r="F73" t="n">
         <v>450</v>
       </c>
-      <c r="G73" t="n">
+      <c r="G73" s="2" t="n">
         <v>37.06</v>
       </c>
       <c r="H73" t="n">
@@ -4235,9 +4239,13 @@
       <c r="I73" t="n">
         <v>32.69</v>
       </c>
-      <c r="J73" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.06 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="b">
@@ -4247,8 +4255,8 @@
       <c r="O73" t="b">
         <v>0</v>
       </c>
-      <c r="P73" t="b">
-        <v>0</v>
+      <c r="P73" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4276,7 +4284,7 @@
       <c r="F74" t="n">
         <v>450</v>
       </c>
-      <c r="G74" t="n">
+      <c r="G74" s="2" t="n">
         <v>36.589</v>
       </c>
       <c r="H74" t="n">
@@ -4285,9 +4293,13 @@
       <c r="I74" t="n">
         <v>34.18</v>
       </c>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.59 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="b">
@@ -4297,8 +4309,8 @@
       <c r="O74" t="b">
         <v>0</v>
       </c>
-      <c r="P74" t="b">
-        <v>0</v>
+      <c r="P74" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -4326,7 +4338,7 @@
       <c r="F75" t="n">
         <v>450</v>
       </c>
-      <c r="G75" t="n">
+      <c r="G75" s="2" t="n">
         <v>36.687</v>
       </c>
       <c r="H75" t="n">
@@ -4335,9 +4347,13 @@
       <c r="I75" t="n">
         <v>31.92</v>
       </c>
-      <c r="J75" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.69 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="b">
@@ -4347,8 +4363,8 @@
       <c r="O75" t="b">
         <v>0</v>
       </c>
-      <c r="P75" t="b">
-        <v>0</v>
+      <c r="P75" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -4376,7 +4392,7 @@
       <c r="F76" t="n">
         <v>450</v>
       </c>
-      <c r="G76" t="n">
+      <c r="G76" s="2" t="n">
         <v>35.932</v>
       </c>
       <c r="H76" t="n">
@@ -4385,9 +4401,13 @@
       <c r="I76" t="n">
         <v>32.08</v>
       </c>
-      <c r="J76" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>over: 35.93 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="b">
@@ -4397,8 +4417,8 @@
       <c r="O76" t="b">
         <v>0</v>
       </c>
-      <c r="P76" t="b">
-        <v>0</v>
+      <c r="P76" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -4426,7 +4446,7 @@
       <c r="F77" t="n">
         <v>450</v>
       </c>
-      <c r="G77" t="n">
+      <c r="G77" s="2" t="n">
         <v>35.448</v>
       </c>
       <c r="H77" t="n">
@@ -4435,9 +4455,13 @@
       <c r="I77" t="n">
         <v>37.23</v>
       </c>
-      <c r="J77" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>over: 35.45 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="b">
@@ -4447,8 +4471,8 @@
       <c r="O77" t="b">
         <v>0</v>
       </c>
-      <c r="P77" t="b">
-        <v>0</v>
+      <c r="P77" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -4476,7 +4500,7 @@
       <c r="F78" t="n">
         <v>450</v>
       </c>
-      <c r="G78" t="n">
+      <c r="G78" s="2" t="n">
         <v>37.013</v>
       </c>
       <c r="H78" t="n">
@@ -4485,9 +4509,13 @@
       <c r="I78" t="n">
         <v>34.98</v>
       </c>
-      <c r="J78" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.01 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="b">
@@ -4497,8 +4525,8 @@
       <c r="O78" t="b">
         <v>0</v>
       </c>
-      <c r="P78" t="b">
-        <v>0</v>
+      <c r="P78" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -4526,7 +4554,7 @@
       <c r="F79" t="n">
         <v>450</v>
       </c>
-      <c r="G79" t="n">
+      <c r="G79" s="2" t="n">
         <v>39.026</v>
       </c>
       <c r="H79" t="n">
@@ -4535,9 +4563,13 @@
       <c r="I79" t="n">
         <v>36.13</v>
       </c>
-      <c r="J79" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>over: 39.03 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="b">
@@ -4547,8 +4579,8 @@
       <c r="O79" t="b">
         <v>0</v>
       </c>
-      <c r="P79" t="b">
-        <v>0</v>
+      <c r="P79" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -4576,7 +4608,7 @@
       <c r="F80" t="n">
         <v>450</v>
       </c>
-      <c r="G80" t="n">
+      <c r="G80" s="2" t="n">
         <v>37.349</v>
       </c>
       <c r="H80" t="n">
@@ -4585,9 +4617,13 @@
       <c r="I80" t="n">
         <v>33.14</v>
       </c>
-      <c r="J80" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.35 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="b">
@@ -4597,8 +4633,8 @@
       <c r="O80" t="b">
         <v>0</v>
       </c>
-      <c r="P80" t="b">
-        <v>0</v>
+      <c r="P80" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -4626,7 +4662,7 @@
       <c r="F81" t="n">
         <v>450</v>
       </c>
-      <c r="G81" t="n">
+      <c r="G81" s="2" t="n">
         <v>36.498</v>
       </c>
       <c r="H81" t="n">
@@ -4635,9 +4671,13 @@
       <c r="I81" t="n">
         <v>34.82</v>
       </c>
-      <c r="J81" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.50 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="b">
@@ -4647,8 +4687,8 @@
       <c r="O81" t="b">
         <v>0</v>
       </c>
-      <c r="P81" t="b">
-        <v>0</v>
+      <c r="P81" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -4676,7 +4716,7 @@
       <c r="F82" t="n">
         <v>450</v>
       </c>
-      <c r="G82" t="n">
+      <c r="G82" s="2" t="n">
         <v>38.493</v>
       </c>
       <c r="H82" t="n">
@@ -4685,9 +4725,13 @@
       <c r="I82" t="n">
         <v>35.05</v>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>over: 38.49 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="b">
@@ -4697,8 +4741,8 @@
       <c r="O82" t="b">
         <v>0</v>
       </c>
-      <c r="P82" t="b">
-        <v>0</v>
+      <c r="P82" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -4726,7 +4770,7 @@
       <c r="F83" t="n">
         <v>450</v>
       </c>
-      <c r="G83" t="n">
+      <c r="G83" s="2" t="n">
         <v>36.384</v>
       </c>
       <c r="H83" t="n">
@@ -4735,9 +4779,13 @@
       <c r="I83" t="n">
         <v>33.45</v>
       </c>
-      <c r="J83" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.38 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="b">
@@ -4747,8 +4795,8 @@
       <c r="O83" t="b">
         <v>0</v>
       </c>
-      <c r="P83" t="b">
-        <v>0</v>
+      <c r="P83" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -4776,7 +4824,7 @@
       <c r="F84" t="n">
         <v>450</v>
       </c>
-      <c r="G84" t="n">
+      <c r="G84" s="2" t="n">
         <v>36.088</v>
       </c>
       <c r="H84" t="n">
@@ -4785,9 +4833,13 @@
       <c r="I84" t="n">
         <v>34.25</v>
       </c>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.09 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="b">
@@ -4797,8 +4849,8 @@
       <c r="O84" t="b">
         <v>0</v>
       </c>
-      <c r="P84" t="b">
-        <v>0</v>
+      <c r="P84" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -4826,7 +4878,7 @@
       <c r="F85" t="n">
         <v>450</v>
       </c>
-      <c r="G85" t="n">
+      <c r="G85" s="2" t="n">
         <v>37.102</v>
       </c>
       <c r="H85" t="n">
@@ -4835,9 +4887,13 @@
       <c r="I85" t="n">
         <v>34.38</v>
       </c>
-      <c r="J85" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.10 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="b">
@@ -4847,8 +4903,8 @@
       <c r="O85" t="b">
         <v>0</v>
       </c>
-      <c r="P85" t="b">
-        <v>0</v>
+      <c r="P85" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -4926,7 +4982,7 @@
       <c r="F87" t="n">
         <v>450</v>
       </c>
-      <c r="G87" t="n">
+      <c r="G87" s="2" t="n">
         <v>39.212</v>
       </c>
       <c r="H87" t="n">
@@ -4935,9 +4991,13 @@
       <c r="I87" t="n">
         <v>35.35</v>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>over: 39.21 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="b">
@@ -4947,8 +5007,8 @@
       <c r="O87" t="b">
         <v>0</v>
       </c>
-      <c r="P87" t="b">
-        <v>0</v>
+      <c r="P87" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -5026,7 +5086,7 @@
       <c r="F89" t="n">
         <v>450</v>
       </c>
-      <c r="G89" t="n">
+      <c r="G89" s="2" t="n">
         <v>36.622</v>
       </c>
       <c r="H89" t="n">
@@ -5035,9 +5095,13 @@
       <c r="I89" t="n">
         <v>34.56</v>
       </c>
-      <c r="J89" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.62 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="b">
@@ -5047,8 +5111,8 @@
       <c r="O89" t="b">
         <v>0</v>
       </c>
-      <c r="P89" t="b">
-        <v>0</v>
+      <c r="P89" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -5076,7 +5140,7 @@
       <c r="F90" t="n">
         <v>450</v>
       </c>
-      <c r="G90" t="n">
+      <c r="G90" s="2" t="n">
         <v>38.416</v>
       </c>
       <c r="H90" t="n">
@@ -5085,9 +5149,13 @@
       <c r="I90" t="n">
         <v>34.91</v>
       </c>
-      <c r="J90" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>over: 38.42 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="b">
@@ -5097,8 +5165,8 @@
       <c r="O90" t="b">
         <v>0</v>
       </c>
-      <c r="P90" t="b">
-        <v>0</v>
+      <c r="P90" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -5126,7 +5194,7 @@
       <c r="F91" t="n">
         <v>450</v>
       </c>
-      <c r="G91" t="n">
+      <c r="G91" s="2" t="n">
         <v>36.058</v>
       </c>
       <c r="H91" t="n">
@@ -5135,9 +5203,13 @@
       <c r="I91" t="n">
         <v>34.86</v>
       </c>
-      <c r="J91" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.06 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="b">
@@ -5147,8 +5219,8 @@
       <c r="O91" t="b">
         <v>0</v>
       </c>
-      <c r="P91" t="b">
-        <v>0</v>
+      <c r="P91" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -5176,7 +5248,7 @@
       <c r="F92" t="n">
         <v>450</v>
       </c>
-      <c r="G92" t="n">
+      <c r="G92" s="2" t="n">
         <v>36.881</v>
       </c>
       <c r="H92" t="n">
@@ -5185,9 +5257,13 @@
       <c r="I92" t="n">
         <v>31.31</v>
       </c>
-      <c r="J92" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.88 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="b">
@@ -5197,8 +5273,8 @@
       <c r="O92" t="b">
         <v>0</v>
       </c>
-      <c r="P92" t="b">
-        <v>0</v>
+      <c r="P92" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -5226,7 +5302,7 @@
       <c r="F93" t="n">
         <v>450</v>
       </c>
-      <c r="G93" t="n">
+      <c r="G93" s="2" t="n">
         <v>37.846</v>
       </c>
       <c r="H93" t="n">
@@ -5235,9 +5311,13 @@
       <c r="I93" t="n">
         <v>34.44</v>
       </c>
-      <c r="J93" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.85 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="b">
@@ -5247,8 +5327,8 @@
       <c r="O93" t="b">
         <v>0</v>
       </c>
-      <c r="P93" t="b">
-        <v>0</v>
+      <c r="P93" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -5276,7 +5356,7 @@
       <c r="F94" t="n">
         <v>450</v>
       </c>
-      <c r="G94" t="n">
+      <c r="G94" s="2" t="n">
         <v>37.461</v>
       </c>
       <c r="H94" t="n">
@@ -5285,9 +5365,13 @@
       <c r="I94" t="n">
         <v>35.47</v>
       </c>
-      <c r="J94" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.46 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="b">
@@ -5297,8 +5381,8 @@
       <c r="O94" t="b">
         <v>0</v>
       </c>
-      <c r="P94" t="b">
-        <v>0</v>
+      <c r="P94" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -5326,7 +5410,7 @@
       <c r="F95" t="n">
         <v>450</v>
       </c>
-      <c r="G95" t="n">
+      <c r="G95" s="2" t="n">
         <v>36.939</v>
       </c>
       <c r="H95" t="n">
@@ -5335,9 +5419,13 @@
       <c r="I95" t="n">
         <v>34.99</v>
       </c>
-      <c r="J95" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.94 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="b">
@@ -5347,8 +5435,8 @@
       <c r="O95" t="b">
         <v>0</v>
       </c>
-      <c r="P95" t="b">
-        <v>0</v>
+      <c r="P95" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -5376,7 +5464,7 @@
       <c r="F96" t="n">
         <v>450</v>
       </c>
-      <c r="G96" t="n">
+      <c r="G96" s="2" t="n">
         <v>40.336</v>
       </c>
       <c r="H96" t="n">
@@ -5385,9 +5473,13 @@
       <c r="I96" t="n">
         <v>35.07</v>
       </c>
-      <c r="J96" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>over: 40.34 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="b">
@@ -5397,8 +5489,8 @@
       <c r="O96" t="b">
         <v>0</v>
       </c>
-      <c r="P96" t="b">
-        <v>0</v>
+      <c r="P96" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -5426,7 +5518,7 @@
       <c r="F97" t="n">
         <v>450</v>
       </c>
-      <c r="G97" t="n">
+      <c r="G97" s="2" t="n">
         <v>37.159</v>
       </c>
       <c r="H97" t="n">
@@ -5435,9 +5527,13 @@
       <c r="I97" t="n">
         <v>29.68</v>
       </c>
-      <c r="J97" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>over: 37.16 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="b">
@@ -5447,8 +5543,8 @@
       <c r="O97" t="b">
         <v>0</v>
       </c>
-      <c r="P97" t="b">
-        <v>0</v>
+      <c r="P97" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -5476,7 +5572,7 @@
       <c r="F98" t="n">
         <v>450</v>
       </c>
-      <c r="G98" t="n">
+      <c r="G98" s="2" t="n">
         <v>36.866</v>
       </c>
       <c r="H98" t="n">
@@ -5485,9 +5581,13 @@
       <c r="I98" t="n">
         <v>34.88</v>
       </c>
-      <c r="J98" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.87 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K98" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="b">
@@ -5497,8 +5597,8 @@
       <c r="O98" t="b">
         <v>0</v>
       </c>
-      <c r="P98" t="b">
-        <v>0</v>
+      <c r="P98" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -5526,7 +5626,7 @@
       <c r="F99" t="n">
         <v>450</v>
       </c>
-      <c r="G99" t="n">
+      <c r="G99" s="2" t="n">
         <v>36.389</v>
       </c>
       <c r="H99" t="n">
@@ -5535,9 +5635,13 @@
       <c r="I99" t="n">
         <v>34.51</v>
       </c>
-      <c r="J99" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>over: 36.39 &gt; 35.0</t>
+        </is>
+      </c>
       <c r="K99" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="b">
@@ -5547,8 +5651,8 @@
       <c r="O99" t="b">
         <v>0</v>
       </c>
-      <c r="P99" t="b">
-        <v>0</v>
+      <c r="P99" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest results (2026-05-19_19-56-12)
</commit_message>
<xml_diff>
--- a/res/csv/data_by_date.xlsx
+++ b/res/csv/data_by_date.xlsx
@@ -4176,7 +4176,7 @@
       <c r="F72" t="n">
         <v>450</v>
       </c>
-      <c r="G72" s="2" t="n">
+      <c r="G72" t="n">
         <v>36.843</v>
       </c>
       <c r="H72" t="n">
@@ -4185,13 +4185,9 @@
       <c r="I72" t="n">
         <v>32.32</v>
       </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.84 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J72" t="inlineStr"/>
       <c r="K72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="b">
@@ -4201,8 +4197,8 @@
       <c r="O72" t="b">
         <v>0</v>
       </c>
-      <c r="P72" s="2" t="b">
-        <v>1</v>
+      <c r="P72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -4230,7 +4226,7 @@
       <c r="F73" t="n">
         <v>450</v>
       </c>
-      <c r="G73" s="2" t="n">
+      <c r="G73" t="n">
         <v>37.06</v>
       </c>
       <c r="H73" t="n">
@@ -4239,13 +4235,9 @@
       <c r="I73" t="n">
         <v>32.69</v>
       </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.06 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J73" t="inlineStr"/>
       <c r="K73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="b">
@@ -4255,8 +4247,8 @@
       <c r="O73" t="b">
         <v>0</v>
       </c>
-      <c r="P73" s="2" t="b">
-        <v>1</v>
+      <c r="P73" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -4284,7 +4276,7 @@
       <c r="F74" t="n">
         <v>450</v>
       </c>
-      <c r="G74" s="2" t="n">
+      <c r="G74" t="n">
         <v>36.589</v>
       </c>
       <c r="H74" t="n">
@@ -4293,13 +4285,9 @@
       <c r="I74" t="n">
         <v>34.18</v>
       </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.59 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J74" t="inlineStr"/>
       <c r="K74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="b">
@@ -4309,8 +4297,8 @@
       <c r="O74" t="b">
         <v>0</v>
       </c>
-      <c r="P74" s="2" t="b">
-        <v>1</v>
+      <c r="P74" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -4338,7 +4326,7 @@
       <c r="F75" t="n">
         <v>450</v>
       </c>
-      <c r="G75" s="2" t="n">
+      <c r="G75" t="n">
         <v>36.687</v>
       </c>
       <c r="H75" t="n">
@@ -4347,13 +4335,9 @@
       <c r="I75" t="n">
         <v>31.92</v>
       </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.69 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J75" t="inlineStr"/>
       <c r="K75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="b">
@@ -4363,8 +4347,8 @@
       <c r="O75" t="b">
         <v>0</v>
       </c>
-      <c r="P75" s="2" t="b">
-        <v>1</v>
+      <c r="P75" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -4392,7 +4376,7 @@
       <c r="F76" t="n">
         <v>450</v>
       </c>
-      <c r="G76" s="2" t="n">
+      <c r="G76" t="n">
         <v>35.932</v>
       </c>
       <c r="H76" t="n">
@@ -4401,13 +4385,9 @@
       <c r="I76" t="n">
         <v>32.08</v>
       </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>over: 35.93 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J76" t="inlineStr"/>
       <c r="K76" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="b">
@@ -4417,8 +4397,8 @@
       <c r="O76" t="b">
         <v>0</v>
       </c>
-      <c r="P76" s="2" t="b">
-        <v>1</v>
+      <c r="P76" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -4446,7 +4426,7 @@
       <c r="F77" t="n">
         <v>450</v>
       </c>
-      <c r="G77" s="2" t="n">
+      <c r="G77" t="n">
         <v>35.448</v>
       </c>
       <c r="H77" t="n">
@@ -4455,13 +4435,9 @@
       <c r="I77" t="n">
         <v>37.23</v>
       </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>over: 35.45 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J77" t="inlineStr"/>
       <c r="K77" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="b">
@@ -4471,8 +4447,8 @@
       <c r="O77" t="b">
         <v>0</v>
       </c>
-      <c r="P77" s="2" t="b">
-        <v>1</v>
+      <c r="P77" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -4500,7 +4476,7 @@
       <c r="F78" t="n">
         <v>450</v>
       </c>
-      <c r="G78" s="2" t="n">
+      <c r="G78" t="n">
         <v>37.013</v>
       </c>
       <c r="H78" t="n">
@@ -4509,13 +4485,9 @@
       <c r="I78" t="n">
         <v>34.98</v>
       </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.01 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J78" t="inlineStr"/>
       <c r="K78" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="b">
@@ -4525,8 +4497,8 @@
       <c r="O78" t="b">
         <v>0</v>
       </c>
-      <c r="P78" s="2" t="b">
-        <v>1</v>
+      <c r="P78" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -4554,7 +4526,7 @@
       <c r="F79" t="n">
         <v>450</v>
       </c>
-      <c r="G79" s="2" t="n">
+      <c r="G79" t="n">
         <v>39.026</v>
       </c>
       <c r="H79" t="n">
@@ -4563,13 +4535,9 @@
       <c r="I79" t="n">
         <v>36.13</v>
       </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>over: 39.03 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J79" t="inlineStr"/>
       <c r="K79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="b">
@@ -4579,8 +4547,8 @@
       <c r="O79" t="b">
         <v>0</v>
       </c>
-      <c r="P79" s="2" t="b">
-        <v>1</v>
+      <c r="P79" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -4608,7 +4576,7 @@
       <c r="F80" t="n">
         <v>450</v>
       </c>
-      <c r="G80" s="2" t="n">
+      <c r="G80" t="n">
         <v>37.349</v>
       </c>
       <c r="H80" t="n">
@@ -4617,13 +4585,9 @@
       <c r="I80" t="n">
         <v>33.14</v>
       </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.35 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J80" t="inlineStr"/>
       <c r="K80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="b">
@@ -4633,8 +4597,8 @@
       <c r="O80" t="b">
         <v>0</v>
       </c>
-      <c r="P80" s="2" t="b">
-        <v>1</v>
+      <c r="P80" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -4662,7 +4626,7 @@
       <c r="F81" t="n">
         <v>450</v>
       </c>
-      <c r="G81" s="2" t="n">
+      <c r="G81" t="n">
         <v>36.498</v>
       </c>
       <c r="H81" t="n">
@@ -4671,13 +4635,9 @@
       <c r="I81" t="n">
         <v>34.82</v>
       </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.50 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J81" t="inlineStr"/>
       <c r="K81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="b">
@@ -4687,8 +4647,8 @@
       <c r="O81" t="b">
         <v>0</v>
       </c>
-      <c r="P81" s="2" t="b">
-        <v>1</v>
+      <c r="P81" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -4716,7 +4676,7 @@
       <c r="F82" t="n">
         <v>450</v>
       </c>
-      <c r="G82" s="2" t="n">
+      <c r="G82" t="n">
         <v>38.493</v>
       </c>
       <c r="H82" t="n">
@@ -4725,13 +4685,9 @@
       <c r="I82" t="n">
         <v>35.05</v>
       </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>over: 38.49 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J82" t="inlineStr"/>
       <c r="K82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="b">
@@ -4741,8 +4697,8 @@
       <c r="O82" t="b">
         <v>0</v>
       </c>
-      <c r="P82" s="2" t="b">
-        <v>1</v>
+      <c r="P82" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -4770,7 +4726,7 @@
       <c r="F83" t="n">
         <v>450</v>
       </c>
-      <c r="G83" s="2" t="n">
+      <c r="G83" t="n">
         <v>36.384</v>
       </c>
       <c r="H83" t="n">
@@ -4779,13 +4735,9 @@
       <c r="I83" t="n">
         <v>33.45</v>
       </c>
-      <c r="J83" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.38 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J83" t="inlineStr"/>
       <c r="K83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="b">
@@ -4795,8 +4747,8 @@
       <c r="O83" t="b">
         <v>0</v>
       </c>
-      <c r="P83" s="2" t="b">
-        <v>1</v>
+      <c r="P83" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -4824,7 +4776,7 @@
       <c r="F84" t="n">
         <v>450</v>
       </c>
-      <c r="G84" s="2" t="n">
+      <c r="G84" t="n">
         <v>36.088</v>
       </c>
       <c r="H84" t="n">
@@ -4833,13 +4785,9 @@
       <c r="I84" t="n">
         <v>34.25</v>
       </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.09 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J84" t="inlineStr"/>
       <c r="K84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="b">
@@ -4849,8 +4797,8 @@
       <c r="O84" t="b">
         <v>0</v>
       </c>
-      <c r="P84" s="2" t="b">
-        <v>1</v>
+      <c r="P84" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -4878,7 +4826,7 @@
       <c r="F85" t="n">
         <v>450</v>
       </c>
-      <c r="G85" s="2" t="n">
+      <c r="G85" t="n">
         <v>37.102</v>
       </c>
       <c r="H85" t="n">
@@ -4887,13 +4835,9 @@
       <c r="I85" t="n">
         <v>34.38</v>
       </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.10 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J85" t="inlineStr"/>
       <c r="K85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="b">
@@ -4903,8 +4847,8 @@
       <c r="O85" t="b">
         <v>0</v>
       </c>
-      <c r="P85" s="2" t="b">
-        <v>1</v>
+      <c r="P85" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -4982,7 +4926,7 @@
       <c r="F87" t="n">
         <v>450</v>
       </c>
-      <c r="G87" s="2" t="n">
+      <c r="G87" t="n">
         <v>39.212</v>
       </c>
       <c r="H87" t="n">
@@ -4991,13 +4935,9 @@
       <c r="I87" t="n">
         <v>35.35</v>
       </c>
-      <c r="J87" s="2" t="inlineStr">
-        <is>
-          <t>over: 39.21 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J87" t="inlineStr"/>
       <c r="K87" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="b">
@@ -5007,8 +4947,8 @@
       <c r="O87" t="b">
         <v>0</v>
       </c>
-      <c r="P87" s="2" t="b">
-        <v>1</v>
+      <c r="P87" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -5086,7 +5026,7 @@
       <c r="F89" t="n">
         <v>450</v>
       </c>
-      <c r="G89" s="2" t="n">
+      <c r="G89" t="n">
         <v>36.622</v>
       </c>
       <c r="H89" t="n">
@@ -5095,13 +5035,9 @@
       <c r="I89" t="n">
         <v>34.56</v>
       </c>
-      <c r="J89" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.62 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J89" t="inlineStr"/>
       <c r="K89" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="b">
@@ -5111,8 +5047,8 @@
       <c r="O89" t="b">
         <v>0</v>
       </c>
-      <c r="P89" s="2" t="b">
-        <v>1</v>
+      <c r="P89" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -5140,7 +5076,7 @@
       <c r="F90" t="n">
         <v>450</v>
       </c>
-      <c r="G90" s="2" t="n">
+      <c r="G90" t="n">
         <v>38.416</v>
       </c>
       <c r="H90" t="n">
@@ -5149,13 +5085,9 @@
       <c r="I90" t="n">
         <v>34.91</v>
       </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t>over: 38.42 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J90" t="inlineStr"/>
       <c r="K90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="b">
@@ -5165,8 +5097,8 @@
       <c r="O90" t="b">
         <v>0</v>
       </c>
-      <c r="P90" s="2" t="b">
-        <v>1</v>
+      <c r="P90" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -5194,7 +5126,7 @@
       <c r="F91" t="n">
         <v>450</v>
       </c>
-      <c r="G91" s="2" t="n">
+      <c r="G91" t="n">
         <v>36.058</v>
       </c>
       <c r="H91" t="n">
@@ -5203,13 +5135,9 @@
       <c r="I91" t="n">
         <v>34.86</v>
       </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.06 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J91" t="inlineStr"/>
       <c r="K91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="b">
@@ -5219,8 +5147,8 @@
       <c r="O91" t="b">
         <v>0</v>
       </c>
-      <c r="P91" s="2" t="b">
-        <v>1</v>
+      <c r="P91" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -5248,7 +5176,7 @@
       <c r="F92" t="n">
         <v>450</v>
       </c>
-      <c r="G92" s="2" t="n">
+      <c r="G92" t="n">
         <v>36.881</v>
       </c>
       <c r="H92" t="n">
@@ -5257,13 +5185,9 @@
       <c r="I92" t="n">
         <v>31.31</v>
       </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.88 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J92" t="inlineStr"/>
       <c r="K92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="b">
@@ -5273,8 +5197,8 @@
       <c r="O92" t="b">
         <v>0</v>
       </c>
-      <c r="P92" s="2" t="b">
-        <v>1</v>
+      <c r="P92" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -5302,7 +5226,7 @@
       <c r="F93" t="n">
         <v>450</v>
       </c>
-      <c r="G93" s="2" t="n">
+      <c r="G93" t="n">
         <v>37.846</v>
       </c>
       <c r="H93" t="n">
@@ -5311,13 +5235,9 @@
       <c r="I93" t="n">
         <v>34.44</v>
       </c>
-      <c r="J93" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.85 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J93" t="inlineStr"/>
       <c r="K93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="b">
@@ -5327,8 +5247,8 @@
       <c r="O93" t="b">
         <v>0</v>
       </c>
-      <c r="P93" s="2" t="b">
-        <v>1</v>
+      <c r="P93" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -5356,7 +5276,7 @@
       <c r="F94" t="n">
         <v>450</v>
       </c>
-      <c r="G94" s="2" t="n">
+      <c r="G94" t="n">
         <v>37.461</v>
       </c>
       <c r="H94" t="n">
@@ -5365,13 +5285,9 @@
       <c r="I94" t="n">
         <v>35.47</v>
       </c>
-      <c r="J94" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.46 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J94" t="inlineStr"/>
       <c r="K94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="b">
@@ -5381,8 +5297,8 @@
       <c r="O94" t="b">
         <v>0</v>
       </c>
-      <c r="P94" s="2" t="b">
-        <v>1</v>
+      <c r="P94" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -5410,7 +5326,7 @@
       <c r="F95" t="n">
         <v>450</v>
       </c>
-      <c r="G95" s="2" t="n">
+      <c r="G95" t="n">
         <v>36.939</v>
       </c>
       <c r="H95" t="n">
@@ -5419,13 +5335,9 @@
       <c r="I95" t="n">
         <v>34.99</v>
       </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.94 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J95" t="inlineStr"/>
       <c r="K95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="b">
@@ -5435,8 +5347,8 @@
       <c r="O95" t="b">
         <v>0</v>
       </c>
-      <c r="P95" s="2" t="b">
-        <v>1</v>
+      <c r="P95" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -5464,7 +5376,7 @@
       <c r="F96" t="n">
         <v>450</v>
       </c>
-      <c r="G96" s="2" t="n">
+      <c r="G96" t="n">
         <v>40.336</v>
       </c>
       <c r="H96" t="n">
@@ -5473,13 +5385,9 @@
       <c r="I96" t="n">
         <v>35.07</v>
       </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t>over: 40.34 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J96" t="inlineStr"/>
       <c r="K96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="b">
@@ -5489,8 +5397,8 @@
       <c r="O96" t="b">
         <v>0</v>
       </c>
-      <c r="P96" s="2" t="b">
-        <v>1</v>
+      <c r="P96" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -5518,7 +5426,7 @@
       <c r="F97" t="n">
         <v>450</v>
       </c>
-      <c r="G97" s="2" t="n">
+      <c r="G97" t="n">
         <v>37.159</v>
       </c>
       <c r="H97" t="n">
@@ -5527,13 +5435,9 @@
       <c r="I97" t="n">
         <v>29.68</v>
       </c>
-      <c r="J97" s="2" t="inlineStr">
-        <is>
-          <t>over: 37.16 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J97" t="inlineStr"/>
       <c r="K97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="b">
@@ -5543,8 +5447,8 @@
       <c r="O97" t="b">
         <v>0</v>
       </c>
-      <c r="P97" s="2" t="b">
-        <v>1</v>
+      <c r="P97" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -5572,7 +5476,7 @@
       <c r="F98" t="n">
         <v>450</v>
       </c>
-      <c r="G98" s="2" t="n">
+      <c r="G98" t="n">
         <v>36.866</v>
       </c>
       <c r="H98" t="n">
@@ -5581,13 +5485,9 @@
       <c r="I98" t="n">
         <v>34.88</v>
       </c>
-      <c r="J98" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.87 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J98" t="inlineStr"/>
       <c r="K98" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="b">
@@ -5597,8 +5497,8 @@
       <c r="O98" t="b">
         <v>0</v>
       </c>
-      <c r="P98" s="2" t="b">
-        <v>1</v>
+      <c r="P98" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -5626,7 +5526,7 @@
       <c r="F99" t="n">
         <v>450</v>
       </c>
-      <c r="G99" s="2" t="n">
+      <c r="G99" t="n">
         <v>36.389</v>
       </c>
       <c r="H99" t="n">
@@ -5635,13 +5535,9 @@
       <c r="I99" t="n">
         <v>34.51</v>
       </c>
-      <c r="J99" s="2" t="inlineStr">
-        <is>
-          <t>over: 36.39 &gt; 35.0</t>
-        </is>
-      </c>
+      <c r="J99" t="inlineStr"/>
       <c r="K99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="b">
@@ -5651,8 +5547,8 @@
       <c r="O99" t="b">
         <v>0</v>
       </c>
-      <c r="P99" s="2" t="b">
-        <v>1</v>
+      <c r="P99" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest results (2026-05-19_20-14-37)
</commit_message>
<xml_diff>
--- a/res/csv/data_by_date.xlsx
+++ b/res/csv/data_by_date.xlsx
@@ -1271,7 +1271,7 @@
         <v>-8.499000000000001</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1555.52</v>
+        <v/>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="b">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>over: 1555.52 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O16" t="b">
@@ -1325,7 +1325,7 @@
         <v>-9.741</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>2122.6</v>
+        <v/>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="b">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>over: 2122.60 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O17" t="b">
@@ -1379,7 +1379,7 @@
         <v>-7.332</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>78633.94</v>
+        <v/>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="b">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>over: 78633.94 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O18" t="b">
@@ -1433,7 +1433,7 @@
         <v>-7.382</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>8247.889999999999</v>
+        <v/>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="b">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>over: 8247.89 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O19" t="b">
@@ -1487,7 +1487,7 @@
         <v>-9.218999999999999</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>31978.97</v>
+        <v/>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="b">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>over: 31978.97 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O20" t="b">
@@ -1541,7 +1541,7 @@
         <v>-7.065</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>4293.41</v>
+        <v/>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="b">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>over: 4293.41 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O21" t="b">
@@ -1595,7 +1595,7 @@
         <v>-8.1</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1062.17</v>
+        <v/>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="b">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>over: 1062.17 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O22" t="b">
@@ -1649,7 +1649,7 @@
         <v>-8.028</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>3053.87</v>
+        <v/>
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="b">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>over: 3053.87 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O23" t="b">
@@ -1703,7 +1703,7 @@
         <v>-6.775</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>23325.19</v>
+        <v/>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="b">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>over: 23325.19 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O24" t="b">
@@ -1757,7 +1757,7 @@
         <v>-6.919</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>4083.92</v>
+        <v/>
       </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="b">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>over: 4083.92 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O25" t="b">
@@ -1811,7 +1811,7 @@
         <v>-7.398</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>3649.45</v>
+        <v/>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="b">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>over: 3649.45 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O26" t="b">
@@ -1865,7 +1865,7 @@
         <v>-6.857</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>2157.59</v>
+        <v/>
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="b">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>over: 2157.59 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O27" t="b">
@@ -1919,7 +1919,7 @@
         <v>-6.436</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>64881.05</v>
+        <v/>
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="b">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>over: 64881.05 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O28" t="b">
@@ -1973,7 +1973,7 @@
         <v>-6.541</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>3778.3</v>
+        <v/>
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="b">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>over: 3778.30 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O29" t="b">
@@ -2027,7 +2027,7 @@
         <v>-8.821</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>5340.69</v>
+        <v/>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="b">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>over: 5340.69 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O30" t="b">
@@ -2081,7 +2081,7 @@
         <v>-9.843</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>17795.66</v>
+        <v/>
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="b">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>over: 17795.66 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O31" t="b">
@@ -2135,7 +2135,7 @@
         <v>-8.044</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>18100.32</v>
+        <v/>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="b">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>over: 18100.32 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O32" t="b">
@@ -2189,7 +2189,7 @@
         <v>-8.036</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>3659.56</v>
+        <v/>
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="b">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>over: 3659.56 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O33" t="b">
@@ -2243,7 +2243,7 @@
         <v>-8.673</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>8031.53</v>
+        <v/>
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="b">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>over: 8031.53 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O34" t="b">
@@ -2297,7 +2297,7 @@
         <v>-6.785</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>16295.7</v>
+        <v/>
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="b">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>over: 16295.70 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O35" t="b">
@@ -2351,7 +2351,7 @@
         <v>-8.525</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>2781.36</v>
+        <v/>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="b">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>over: 2781.36 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O36" t="b">
@@ -2405,7 +2405,7 @@
         <v>-8.239000000000001</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>2688.22</v>
+        <v/>
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="b">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>over: 2688.22 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O37" t="b">
@@ -2459,7 +2459,7 @@
         <v>-6.785</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>8688.93</v>
+        <v/>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="b">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>over: 8688.93 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O38" t="b">
@@ -2513,7 +2513,7 @@
         <v>-6.643</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>46254.71</v>
+        <v/>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="b">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>over: 46254.71 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O39" t="b">
@@ -2567,7 +2567,7 @@
         <v>-7.891</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>1429.78</v>
+        <v/>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="b">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>over: 1429.78 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O40" t="b">
@@ -2621,7 +2621,7 @@
         <v>-6.389</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>5666.98</v>
+        <v/>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="b">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>over: 5666.98 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O41" t="b">
@@ -2675,7 +2675,7 @@
         <v>-7.481</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>5615.99</v>
+        <v/>
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="b">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>over: 5615.99 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O42" t="b">
@@ -2729,7 +2729,7 @@
         <v>-7.55</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>7012.52</v>
+        <v/>
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="b">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>over: 7012.52 &gt; 60.0</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="O43" t="b">
@@ -4327,7 +4327,7 @@
         <v>450</v>
       </c>
       <c r="G75" t="n">
-        <v>36.687</v>
+        <v>37.113</v>
       </c>
       <c r="H75" t="n">
         <v>-12.083</v>
@@ -4477,7 +4477,7 @@
         <v>450</v>
       </c>
       <c r="G78" t="n">
-        <v>37.013</v>
+        <v>37.911</v>
       </c>
       <c r="H78" t="n">
         <v>-10.763</v>
@@ -4727,7 +4727,7 @@
         <v>450</v>
       </c>
       <c r="G83" t="n">
-        <v>36.384</v>
+        <v>39.186</v>
       </c>
       <c r="H83" t="n">
         <v>-9.867000000000001</v>
@@ -4777,7 +4777,7 @@
         <v>450</v>
       </c>
       <c r="G84" t="n">
-        <v>36.088</v>
+        <v>36.272</v>
       </c>
       <c r="H84" t="n">
         <v>-11.982</v>
@@ -4977,7 +4977,7 @@
         <v>450</v>
       </c>
       <c r="G88" t="n">
-        <v>32.319</v>
+        <v>38.696</v>
       </c>
       <c r="H88" t="n">
         <v>-9.875</v>
@@ -5027,7 +5027,7 @@
         <v>450</v>
       </c>
       <c r="G89" t="n">
-        <v>36.622</v>
+        <v>36.72</v>
       </c>
       <c r="H89" t="n">
         <v>-12.361</v>
@@ -5127,7 +5127,7 @@
         <v>450</v>
       </c>
       <c r="G91" t="n">
-        <v>36.058</v>
+        <v>36.597</v>
       </c>
       <c r="H91" t="n">
         <v>-10.028</v>
@@ -5227,7 +5227,7 @@
         <v>450</v>
       </c>
       <c r="G93" t="n">
-        <v>37.846</v>
+        <v>38.014</v>
       </c>
       <c r="H93" t="n">
         <v>-11.385</v>
@@ -5277,7 +5277,7 @@
         <v>450</v>
       </c>
       <c r="G94" t="n">
-        <v>37.461</v>
+        <v>37.603</v>
       </c>
       <c r="H94" t="n">
         <v>-10.471</v>
@@ -5477,7 +5477,7 @@
         <v>450</v>
       </c>
       <c r="G98" t="n">
-        <v>36.866</v>
+        <v>37.279</v>
       </c>
       <c r="H98" t="n">
         <v>-10.442</v>

</xml_diff>

<commit_message>
Update latest results (2026-05-19_20-17-52)
</commit_message>
<xml_diff>
--- a/res/csv/data_by_date.xlsx
+++ b/res/csv/data_by_date.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:Q99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -448,13 +448,14 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,35 +506,40 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>dlam_dV_pm_per_V</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>reason_ER_dB</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_ER_dB</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>reason_IL_dB</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_IL_dB</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>reason_Vpi_V</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_Vpi_V</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>is_problematic</t>
         </is>
@@ -573,19 +579,22 @@
       <c r="I2" t="n">
         <v>26.78</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="b">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
+      <c r="J2" t="n">
+        <v>-180.3</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -623,19 +632,22 @@
       <c r="I3" t="n">
         <v>29.32</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
+      <c r="J3" t="n">
+        <v>-166.8</v>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -673,19 +685,22 @@
       <c r="I4" t="n">
         <v>29.5</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
+      <c r="J4" t="n">
+        <v>-166.41</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -723,19 +738,22 @@
       <c r="I5" t="n">
         <v>26.46</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
+      <c r="J5" t="n">
+        <v>-186.65</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -773,19 +791,22 @@
       <c r="I6" t="n">
         <v>28.49</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="b">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="b">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
+      <c r="J6" t="n">
+        <v>-172.51</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -823,19 +844,22 @@
       <c r="I7" t="n">
         <v>30.46</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="b">
-        <v>0</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
+      <c r="J7" t="n">
+        <v>-161.57</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -873,19 +897,22 @@
       <c r="I8" t="n">
         <v>26.34</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="b">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="b">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
+      <c r="J8" t="n">
+        <v>-186.21</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -923,19 +950,22 @@
       <c r="I9" t="n">
         <v>27.28</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="b">
-        <v>0</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="b">
-        <v>0</v>
-      </c>
+      <c r="J9" t="n">
+        <v>-179.2</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -973,19 +1003,22 @@
       <c r="I10" t="n">
         <v>30.36</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="b">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="b">
-        <v>0</v>
-      </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="b">
-        <v>0</v>
-      </c>
+      <c r="J10" t="n">
+        <v>-162.44</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1023,19 +1056,22 @@
       <c r="I11" t="n">
         <v>27.58</v>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="b">
-        <v>0</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="b">
-        <v>0</v>
-      </c>
+      <c r="J11" t="n">
+        <v>-178.67</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1073,19 +1109,22 @@
       <c r="I12" t="n">
         <v>28.1</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="b">
-        <v>0</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="b">
-        <v>0</v>
-      </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="b">
-        <v>0</v>
-      </c>
+      <c r="J12" t="n">
+        <v>-173.13</v>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1123,19 +1162,22 @@
       <c r="I13" t="n">
         <v>27.81</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="b">
-        <v>0</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="b">
-        <v>0</v>
-      </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="b">
-        <v>0</v>
-      </c>
+      <c r="J13" t="n">
+        <v>-177.9</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="b">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1173,19 +1215,22 @@
       <c r="I14" t="n">
         <v>27.6</v>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="b">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="b">
-        <v>0</v>
-      </c>
+      <c r="J14" t="n">
+        <v>-178.79</v>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1223,19 +1268,22 @@
       <c r="I15" t="n">
         <v>28.74</v>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="b">
-        <v>0</v>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="b">
-        <v>0</v>
-      </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="b">
-        <v>0</v>
-      </c>
+      <c r="J15" t="n">
+        <v>-169.78</v>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1273,23 +1321,26 @@
       <c r="I16" s="2" t="n">
         <v/>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="b">
-        <v>0</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O16" t="b">
+      <c r="J16" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=3.13 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P16" t="b">
         <v>1</v>
       </c>
-      <c r="P16" s="2" t="b">
+      <c r="Q16" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1327,23 +1378,26 @@
       <c r="I17" s="2" t="n">
         <v/>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="b">
-        <v>0</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O17" t="b">
+      <c r="J17" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=2.30 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P17" t="b">
         <v>1</v>
       </c>
-      <c r="P17" s="2" t="b">
+      <c r="Q17" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1381,23 +1435,26 @@
       <c r="I18" s="2" t="n">
         <v/>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="b">
-        <v>0</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O18" t="b">
+      <c r="J18" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.06 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P18" t="b">
         <v>1</v>
       </c>
-      <c r="P18" s="2" t="b">
+      <c r="Q18" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1435,23 +1492,26 @@
       <c r="I19" s="2" t="n">
         <v/>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="b">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="b">
-        <v>0</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O19" t="b">
+      <c r="J19" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="b">
+        <v>0</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.59 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P19" t="b">
         <v>1</v>
       </c>
-      <c r="P19" s="2" t="b">
+      <c r="Q19" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1489,23 +1549,26 @@
       <c r="I20" s="2" t="n">
         <v/>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="b">
-        <v>0</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="b">
-        <v>0</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O20" t="b">
+      <c r="J20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.15 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P20" t="b">
         <v>1</v>
       </c>
-      <c r="P20" s="2" t="b">
+      <c r="Q20" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1543,23 +1606,26 @@
       <c r="I21" s="2" t="n">
         <v/>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="b">
-        <v>0</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O21" t="b">
+      <c r="J21" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="b">
+        <v>0</v>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="b">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.16 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P21" t="b">
         <v>1</v>
       </c>
-      <c r="P21" s="2" t="b">
+      <c r="Q21" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1597,23 +1663,26 @@
       <c r="I22" s="2" t="n">
         <v/>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="b">
-        <v>0</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="b">
-        <v>0</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O22" t="b">
+      <c r="J22" t="n">
+        <v>-4.66</v>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="b">
+        <v>0</v>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=4.66 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P22" t="b">
         <v>1</v>
       </c>
-      <c r="P22" s="2" t="b">
+      <c r="Q22" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1651,23 +1720,26 @@
       <c r="I23" s="2" t="n">
         <v/>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="b">
-        <v>0</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O23" t="b">
+      <c r="J23" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="b">
+        <v>0</v>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.61 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P23" t="b">
         <v>1</v>
       </c>
-      <c r="P23" s="2" t="b">
+      <c r="Q23" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1705,23 +1777,26 @@
       <c r="I24" s="2" t="n">
         <v/>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="b">
-        <v>0</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="b">
-        <v>0</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O24" t="b">
+      <c r="J24" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.21 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P24" t="b">
         <v>1</v>
       </c>
-      <c r="P24" s="2" t="b">
+      <c r="Q24" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1759,23 +1834,26 @@
       <c r="I25" s="2" t="n">
         <v/>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O25" t="b">
+      <c r="J25" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.20 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P25" t="b">
         <v>1</v>
       </c>
-      <c r="P25" s="2" t="b">
+      <c r="Q25" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1813,23 +1891,26 @@
       <c r="I26" s="2" t="n">
         <v/>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="b">
-        <v>0</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="b">
-        <v>0</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O26" t="b">
+      <c r="J26" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.35 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P26" t="b">
         <v>1</v>
       </c>
-      <c r="P26" s="2" t="b">
+      <c r="Q26" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1867,23 +1948,26 @@
       <c r="I27" s="2" t="n">
         <v/>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="b">
-        <v>0</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="b">
-        <v>0</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O27" t="b">
+      <c r="J27" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=2.31 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P27" t="b">
         <v>1</v>
       </c>
-      <c r="P27" s="2" t="b">
+      <c r="Q27" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1921,23 +2005,26 @@
       <c r="I28" s="2" t="n">
         <v/>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="b">
-        <v>0</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="b">
-        <v>0</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O28" t="b">
+      <c r="J28" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="b">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.08 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P28" t="b">
         <v>1</v>
       </c>
-      <c r="P28" s="2" t="b">
+      <c r="Q28" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1975,23 +2062,26 @@
       <c r="I29" s="2" t="n">
         <v/>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="b">
-        <v>0</v>
-      </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="b">
-        <v>0</v>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O29" t="b">
+      <c r="J29" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="b">
+        <v>0</v>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.30 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P29" t="b">
         <v>1</v>
       </c>
-      <c r="P29" s="2" t="b">
+      <c r="Q29" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2029,23 +2119,26 @@
       <c r="I30" s="2" t="n">
         <v/>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="b">
-        <v>0</v>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="b">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O30" t="b">
+      <c r="J30" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="b">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.91 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P30" t="b">
         <v>1</v>
       </c>
-      <c r="P30" s="2" t="b">
+      <c r="Q30" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2083,23 +2176,26 @@
       <c r="I31" s="2" t="n">
         <v/>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="b">
-        <v>0</v>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="b">
-        <v>0</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O31" t="b">
+      <c r="J31" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="b">
+        <v>0</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.28 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P31" t="b">
         <v>1</v>
       </c>
-      <c r="P31" s="2" t="b">
+      <c r="Q31" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2137,23 +2233,26 @@
       <c r="I32" s="2" t="n">
         <v/>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="b">
-        <v>0</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="b">
-        <v>0</v>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O32" t="b">
+      <c r="J32" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.27 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P32" t="b">
         <v>1</v>
       </c>
-      <c r="P32" s="2" t="b">
+      <c r="Q32" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2191,23 +2290,26 @@
       <c r="I33" s="2" t="n">
         <v/>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="b">
-        <v>0</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="b">
-        <v>0</v>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O33" t="b">
+      <c r="J33" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.33 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P33" t="b">
         <v>1</v>
       </c>
-      <c r="P33" s="2" t="b">
+      <c r="Q33" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2245,23 +2347,26 @@
       <c r="I34" s="2" t="n">
         <v/>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="b">
-        <v>0</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="b">
-        <v>0</v>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O34" t="b">
+      <c r="J34" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="b">
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="b">
+        <v>0</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.61 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P34" t="b">
         <v>1</v>
       </c>
-      <c r="P34" s="2" t="b">
+      <c r="Q34" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2299,23 +2404,26 @@
       <c r="I35" s="2" t="n">
         <v/>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="b">
-        <v>0</v>
-      </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="b">
-        <v>0</v>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O35" t="b">
+      <c r="J35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="b">
+        <v>0</v>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="b">
+        <v>0</v>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.30 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P35" t="b">
         <v>1</v>
       </c>
-      <c r="P35" s="2" t="b">
+      <c r="Q35" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2353,23 +2461,26 @@
       <c r="I36" s="2" t="n">
         <v/>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="b">
-        <v>0</v>
-      </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="b">
-        <v>0</v>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O36" t="b">
+      <c r="J36" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="b">
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="b">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.76 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P36" t="b">
         <v>1</v>
       </c>
-      <c r="P36" s="2" t="b">
+      <c r="Q36" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2407,23 +2518,26 @@
       <c r="I37" s="2" t="n">
         <v/>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="b">
-        <v>0</v>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="b">
-        <v>0</v>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O37" t="b">
+      <c r="J37" t="n">
+        <v>-1.84</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="b">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="b">
+        <v>0</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=1.84 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P37" t="b">
         <v>1</v>
       </c>
-      <c r="P37" s="2" t="b">
+      <c r="Q37" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2461,23 +2575,26 @@
       <c r="I38" s="2" t="n">
         <v/>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="b">
-        <v>0</v>
-      </c>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="b">
-        <v>0</v>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O38" t="b">
+      <c r="J38" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="b">
+        <v>0</v>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="b">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.57 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P38" t="b">
         <v>1</v>
       </c>
-      <c r="P38" s="2" t="b">
+      <c r="Q38" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2515,23 +2632,26 @@
       <c r="I39" s="2" t="n">
         <v/>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="b">
-        <v>0</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="b">
-        <v>0</v>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O39" t="b">
+      <c r="J39" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="b">
+        <v>0</v>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="b">
+        <v>0</v>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.11 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P39" t="b">
         <v>1</v>
       </c>
-      <c r="P39" s="2" t="b">
+      <c r="Q39" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2569,23 +2689,26 @@
       <c r="I40" s="2" t="n">
         <v/>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="b">
-        <v>0</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="b">
-        <v>0</v>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O40" t="b">
+      <c r="J40" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="b">
+        <v>0</v>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="b">
+        <v>0</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=3.44 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P40" t="b">
         <v>1</v>
       </c>
-      <c r="P40" s="2" t="b">
+      <c r="Q40" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2623,23 +2746,26 @@
       <c r="I41" s="2" t="n">
         <v/>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="b">
-        <v>0</v>
-      </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="b">
-        <v>0</v>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O41" t="b">
+      <c r="J41" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="b">
+        <v>0</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="b">
+        <v>0</v>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.87 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P41" t="b">
         <v>1</v>
       </c>
-      <c r="P41" s="2" t="b">
+      <c r="Q41" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2677,23 +2803,26 @@
       <c r="I42" s="2" t="n">
         <v/>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="b">
-        <v>0</v>
-      </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="b">
-        <v>0</v>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O42" t="b">
+      <c r="J42" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="b">
+        <v>0</v>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="b">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.88 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P42" t="b">
         <v>1</v>
       </c>
-      <c r="P42" s="2" t="b">
+      <c r="Q42" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2731,23 +2860,26 @@
       <c r="I43" s="2" t="n">
         <v/>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="b">
-        <v>0</v>
-      </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="b">
-        <v>0</v>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="O43" t="b">
+      <c r="J43" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="b">
+        <v>0</v>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV|=0.71 &lt; 10 pm/V (slope filter)</t>
+        </is>
+      </c>
+      <c r="P43" t="b">
         <v>1</v>
       </c>
-      <c r="P43" s="2" t="b">
+      <c r="Q43" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2785,19 +2917,22 @@
       <c r="I44" t="n">
         <v>36.18</v>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="b">
-        <v>0</v>
-      </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="b">
-        <v>0</v>
-      </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="b">
-        <v>0</v>
-      </c>
+      <c r="J44" t="n">
+        <v>-133.85</v>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="b">
+        <v>0</v>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="b">
+        <v>0</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
       <c r="P44" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2835,19 +2970,22 @@
       <c r="I45" t="n">
         <v>42.12</v>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="b">
-        <v>0</v>
-      </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="b">
-        <v>0</v>
-      </c>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="b">
-        <v>0</v>
-      </c>
+      <c r="J45" t="n">
+        <v>-116.09</v>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="b">
+        <v>0</v>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="b">
+        <v>0</v>
+      </c>
+      <c r="O45" t="inlineStr"/>
       <c r="P45" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2885,19 +3023,22 @@
       <c r="I46" t="n">
         <v>42.05</v>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="b">
-        <v>0</v>
-      </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="b">
-        <v>0</v>
-      </c>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="b">
-        <v>0</v>
-      </c>
+      <c r="J46" t="n">
+        <v>-116.4</v>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="b">
+        <v>0</v>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="b">
+        <v>0</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
       <c r="P46" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2935,19 +3076,22 @@
       <c r="I47" t="n">
         <v>35.49</v>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="b">
-        <v>0</v>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="b">
-        <v>0</v>
-      </c>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="b">
-        <v>0</v>
-      </c>
+      <c r="J47" t="n">
+        <v>-137.06</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="b">
+        <v>0</v>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="b">
+        <v>0</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2985,19 +3129,22 @@
       <c r="I48" t="n">
         <v>45.89</v>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="b">
-        <v>0</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="b">
-        <v>0</v>
-      </c>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="b">
-        <v>0</v>
-      </c>
+      <c r="J48" t="n">
+        <v>-107.06</v>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="b">
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="b">
+        <v>0</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
       <c r="P48" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3035,19 +3182,22 @@
       <c r="I49" t="n">
         <v>44.36</v>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="b">
-        <v>0</v>
-      </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="b">
-        <v>0</v>
-      </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="b">
-        <v>0</v>
-      </c>
+      <c r="J49" t="n">
+        <v>-112.21</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="b">
+        <v>0</v>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="b">
+        <v>0</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3085,19 +3235,22 @@
       <c r="I50" t="n">
         <v>35.16</v>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="b">
-        <v>0</v>
-      </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="b">
-        <v>0</v>
-      </c>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="b">
-        <v>0</v>
-      </c>
+      <c r="J50" t="n">
+        <v>-140.86</v>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="b">
+        <v>0</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
       <c r="P50" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3135,19 +3288,22 @@
       <c r="I51" t="n">
         <v>38.29</v>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="b">
-        <v>0</v>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="b">
-        <v>0</v>
-      </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="b">
-        <v>0</v>
-      </c>
+      <c r="J51" t="n">
+        <v>-128.09</v>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="b">
+        <v>0</v>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="b">
+        <v>0</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
       <c r="P51" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3185,19 +3341,22 @@
       <c r="I52" t="n">
         <v>46.64</v>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="b">
-        <v>0</v>
-      </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="b">
-        <v>0</v>
-      </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="b">
-        <v>0</v>
-      </c>
+      <c r="J52" t="n">
+        <v>-106.92</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="b">
+        <v>0</v>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="b">
+        <v>0</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
       <c r="P52" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3235,19 +3394,22 @@
       <c r="I53" t="n">
         <v>40.54</v>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="b">
-        <v>0</v>
-      </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="b">
-        <v>0</v>
-      </c>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="b">
-        <v>0</v>
-      </c>
+      <c r="J53" t="n">
+        <v>-120.67</v>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="b">
+        <v>0</v>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="b">
+        <v>0</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
       <c r="P53" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3285,19 +3447,22 @@
       <c r="I54" t="n">
         <v>37.81</v>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="b">
-        <v>0</v>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="b">
-        <v>0</v>
-      </c>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="b">
-        <v>0</v>
-      </c>
+      <c r="J54" t="n">
+        <v>-130.6</v>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="b">
+        <v>0</v>
+      </c>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="b">
+        <v>0</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
       <c r="P54" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3335,19 +3500,22 @@
       <c r="I55" t="n">
         <v>42.12</v>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="b">
-        <v>0</v>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="b">
-        <v>0</v>
-      </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="b">
-        <v>0</v>
-      </c>
+      <c r="J55" t="n">
+        <v>-118.08</v>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="b">
+        <v>0</v>
+      </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="b">
+        <v>0</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
       <c r="P55" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3385,19 +3553,22 @@
       <c r="I56" t="n">
         <v>42.37</v>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="b">
-        <v>0</v>
-      </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="b">
-        <v>0</v>
-      </c>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="b">
-        <v>0</v>
-      </c>
+      <c r="J56" t="n">
+        <v>-115.51</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="b">
+        <v>0</v>
+      </c>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="b">
+        <v>0</v>
+      </c>
+      <c r="O56" t="inlineStr"/>
       <c r="P56" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3435,19 +3606,22 @@
       <c r="I57" t="n">
         <v>37.93</v>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="b">
-        <v>0</v>
-      </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="b">
-        <v>0</v>
-      </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="b">
-        <v>0</v>
-      </c>
+      <c r="J57" t="n">
+        <v>-129.17</v>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="b">
+        <v>0</v>
+      </c>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="b">
+        <v>0</v>
+      </c>
+      <c r="O57" t="inlineStr"/>
       <c r="P57" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3485,19 +3659,22 @@
       <c r="I58" t="n">
         <v>41.34</v>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="b">
-        <v>0</v>
-      </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="b">
-        <v>0</v>
-      </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="b">
-        <v>0</v>
-      </c>
+      <c r="J58" t="n">
+        <v>-118.03</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="b">
+        <v>0</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
       <c r="P58" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q58" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3535,19 +3712,22 @@
       <c r="I59" t="n">
         <v>37.35</v>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="b">
-        <v>0</v>
-      </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="b">
-        <v>0</v>
-      </c>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="b">
-        <v>0</v>
-      </c>
+      <c r="J59" t="n">
+        <v>-130.75</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="b">
+        <v>0</v>
+      </c>
+      <c r="O59" t="inlineStr"/>
       <c r="P59" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3585,19 +3765,22 @@
       <c r="I60" t="n">
         <v>38.19</v>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="b">
-        <v>0</v>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="b">
-        <v>0</v>
-      </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="b">
-        <v>0</v>
-      </c>
+      <c r="J60" t="n">
+        <v>-127.31</v>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="b">
+        <v>0</v>
+      </c>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="b">
+        <v>0</v>
+      </c>
+      <c r="O60" t="inlineStr"/>
       <c r="P60" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q60" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3635,19 +3818,22 @@
       <c r="I61" t="n">
         <v>40.4</v>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="b">
-        <v>0</v>
-      </c>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="b">
-        <v>0</v>
-      </c>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="b">
-        <v>0</v>
-      </c>
+      <c r="J61" t="n">
+        <v>-121.69</v>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="b">
+        <v>0</v>
+      </c>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="b">
+        <v>0</v>
+      </c>
+      <c r="O61" t="inlineStr"/>
       <c r="P61" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q61" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3685,19 +3871,22 @@
       <c r="I62" t="n">
         <v>39.5</v>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="b">
-        <v>0</v>
-      </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="b">
-        <v>0</v>
-      </c>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="b">
-        <v>0</v>
-      </c>
+      <c r="J62" t="n">
+        <v>-123.84</v>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="b">
+        <v>0</v>
+      </c>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="b">
+        <v>0</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
       <c r="P62" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q62" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3735,19 +3924,22 @@
       <c r="I63" t="n">
         <v>44.23</v>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="b">
-        <v>0</v>
-      </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="b">
-        <v>0</v>
-      </c>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="b">
-        <v>0</v>
-      </c>
+      <c r="J63" t="n">
+        <v>-111.39</v>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="b">
+        <v>0</v>
+      </c>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="b">
+        <v>0</v>
+      </c>
+      <c r="O63" t="inlineStr"/>
       <c r="P63" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q63" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3785,19 +3977,22 @@
       <c r="I64" t="n">
         <v>38.16</v>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="b">
-        <v>0</v>
-      </c>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="b">
-        <v>0</v>
-      </c>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="b">
-        <v>0</v>
-      </c>
+      <c r="J64" t="n">
+        <v>-128.72</v>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="b">
+        <v>0</v>
+      </c>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="b">
+        <v>0</v>
+      </c>
+      <c r="O64" t="inlineStr"/>
       <c r="P64" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q64" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3835,19 +4030,22 @@
       <c r="I65" t="n">
         <v>42.95</v>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="b">
-        <v>0</v>
-      </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="b">
-        <v>0</v>
-      </c>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="b">
-        <v>0</v>
-      </c>
+      <c r="J65" t="n">
+        <v>-113.59</v>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="b">
+        <v>0</v>
+      </c>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="b">
+        <v>0</v>
+      </c>
+      <c r="O65" t="inlineStr"/>
       <c r="P65" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3885,19 +4083,22 @@
       <c r="I66" t="n">
         <v>43.37</v>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="b">
-        <v>0</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="b">
-        <v>0</v>
-      </c>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="b">
-        <v>0</v>
-      </c>
+      <c r="J66" t="n">
+        <v>-114.23</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="b">
+        <v>0</v>
+      </c>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="b">
+        <v>0</v>
+      </c>
+      <c r="O66" t="inlineStr"/>
       <c r="P66" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3935,19 +4136,22 @@
       <c r="I67" t="n">
         <v>41.84</v>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="b">
-        <v>0</v>
-      </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="b">
-        <v>0</v>
-      </c>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="b">
-        <v>0</v>
-      </c>
+      <c r="J67" t="n">
+        <v>-117.58</v>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="b">
+        <v>0</v>
+      </c>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="b">
+        <v>0</v>
+      </c>
+      <c r="O67" t="inlineStr"/>
       <c r="P67" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q67" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3985,19 +4189,22 @@
       <c r="I68" t="n">
         <v>40.19</v>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="b">
-        <v>0</v>
-      </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="b">
-        <v>0</v>
-      </c>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="b">
-        <v>0</v>
-      </c>
+      <c r="J68" t="n">
+        <v>-121.84</v>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="b">
+        <v>0</v>
+      </c>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="b">
+        <v>0</v>
+      </c>
+      <c r="O68" t="inlineStr"/>
       <c r="P68" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4035,19 +4242,22 @@
       <c r="I69" t="n">
         <v>45.97</v>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="b">
-        <v>0</v>
-      </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="b">
-        <v>0</v>
-      </c>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="b">
-        <v>0</v>
-      </c>
+      <c r="J69" t="n">
+        <v>-107.66</v>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="b">
+        <v>0</v>
+      </c>
+      <c r="O69" t="inlineStr"/>
       <c r="P69" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4085,19 +4295,22 @@
       <c r="I70" t="n">
         <v>43.91</v>
       </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="b">
-        <v>0</v>
-      </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="b">
-        <v>0</v>
-      </c>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="b">
-        <v>0</v>
-      </c>
+      <c r="J70" t="n">
+        <v>-112.15</v>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="b">
+        <v>0</v>
+      </c>
+      <c r="O70" t="inlineStr"/>
       <c r="P70" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4135,19 +4348,22 @@
       <c r="I71" t="n">
         <v>40.04</v>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="b">
-        <v>0</v>
-      </c>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="b">
-        <v>0</v>
-      </c>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="b">
-        <v>0</v>
-      </c>
+      <c r="J71" t="n">
+        <v>-123.04</v>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="b">
+        <v>0</v>
+      </c>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="b">
+        <v>0</v>
+      </c>
+      <c r="O71" t="inlineStr"/>
       <c r="P71" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4185,19 +4401,22 @@
       <c r="I72" t="n">
         <v>32.32</v>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="b">
-        <v>0</v>
-      </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="b">
-        <v>0</v>
-      </c>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="b">
-        <v>0</v>
-      </c>
+      <c r="J72" t="n">
+        <v>-220.01</v>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="b">
+        <v>0</v>
+      </c>
+      <c r="O72" t="inlineStr"/>
       <c r="P72" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4235,19 +4454,22 @@
       <c r="I73" t="n">
         <v>32.69</v>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="b">
-        <v>0</v>
-      </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="b">
-        <v>0</v>
-      </c>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="b">
-        <v>0</v>
-      </c>
+      <c r="J73" t="n">
+        <v>-218.92</v>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="b">
+        <v>0</v>
+      </c>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="b">
+        <v>0</v>
+      </c>
+      <c r="O73" t="inlineStr"/>
       <c r="P73" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q73" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4285,19 +4507,22 @@
       <c r="I74" t="n">
         <v>34.18</v>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="b">
-        <v>0</v>
-      </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="b">
-        <v>0</v>
-      </c>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="b">
-        <v>0</v>
-      </c>
+      <c r="J74" t="n">
+        <v>-208.32</v>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="b">
+        <v>0</v>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="b">
+        <v>0</v>
+      </c>
+      <c r="O74" t="inlineStr"/>
       <c r="P74" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4335,19 +4560,22 @@
       <c r="I75" t="n">
         <v>31.92</v>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="b">
-        <v>0</v>
-      </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="b">
-        <v>0</v>
-      </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="b">
-        <v>0</v>
-      </c>
+      <c r="J75" t="n">
+        <v>-222.17</v>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="b">
+        <v>0</v>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="b">
+        <v>0</v>
+      </c>
+      <c r="O75" t="inlineStr"/>
       <c r="P75" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4385,19 +4613,22 @@
       <c r="I76" t="n">
         <v>32.08</v>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="b">
-        <v>0</v>
-      </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="b">
-        <v>0</v>
-      </c>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="b">
-        <v>0</v>
-      </c>
+      <c r="J76" t="n">
+        <v>-224.07</v>
+      </c>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="b">
+        <v>0</v>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="b">
+        <v>0</v>
+      </c>
+      <c r="O76" t="inlineStr"/>
       <c r="P76" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4435,19 +4666,22 @@
       <c r="I77" t="n">
         <v>37.23</v>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="b">
-        <v>0</v>
-      </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="b">
-        <v>0</v>
-      </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="b">
-        <v>0</v>
-      </c>
+      <c r="J77" t="n">
+        <v>-191.68</v>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="b">
+        <v>0</v>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="b">
+        <v>0</v>
+      </c>
+      <c r="O77" t="inlineStr"/>
       <c r="P77" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4485,19 +4719,22 @@
       <c r="I78" t="n">
         <v>34.98</v>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="b">
-        <v>0</v>
-      </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="b">
-        <v>0</v>
-      </c>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="b">
-        <v>0</v>
-      </c>
+      <c r="J78" t="n">
+        <v>-202.41</v>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="b">
+        <v>0</v>
+      </c>
+      <c r="O78" t="inlineStr"/>
       <c r="P78" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q78" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4535,19 +4772,22 @@
       <c r="I79" t="n">
         <v>36.13</v>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="b">
-        <v>0</v>
-      </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="b">
-        <v>0</v>
-      </c>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="b">
-        <v>0</v>
-      </c>
+      <c r="J79" t="n">
+        <v>-199.12</v>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="b">
+        <v>0</v>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="b">
+        <v>0</v>
+      </c>
+      <c r="O79" t="inlineStr"/>
       <c r="P79" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4585,19 +4825,22 @@
       <c r="I80" t="n">
         <v>33.14</v>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="b">
-        <v>0</v>
-      </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="b">
-        <v>0</v>
-      </c>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="b">
-        <v>0</v>
-      </c>
+      <c r="J80" t="n">
+        <v>-214.56</v>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="b">
+        <v>0</v>
+      </c>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="b">
+        <v>0</v>
+      </c>
+      <c r="O80" t="inlineStr"/>
       <c r="P80" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4635,19 +4878,22 @@
       <c r="I81" t="n">
         <v>34.82</v>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="b">
-        <v>0</v>
-      </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="b">
-        <v>0</v>
-      </c>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="b">
-        <v>0</v>
-      </c>
+      <c r="J81" t="n">
+        <v>-204.04</v>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="b">
+        <v>0</v>
+      </c>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="b">
+        <v>0</v>
+      </c>
+      <c r="O81" t="inlineStr"/>
       <c r="P81" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4685,19 +4931,22 @@
       <c r="I82" t="n">
         <v>35.05</v>
       </c>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="b">
-        <v>0</v>
-      </c>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="b">
-        <v>0</v>
-      </c>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="b">
-        <v>0</v>
-      </c>
+      <c r="J82" t="n">
+        <v>-203.22</v>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="b">
+        <v>0</v>
+      </c>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="b">
+        <v>0</v>
+      </c>
+      <c r="O82" t="inlineStr"/>
       <c r="P82" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4735,19 +4984,22 @@
       <c r="I83" t="n">
         <v>33.45</v>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="b">
-        <v>0</v>
-      </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="b">
-        <v>0</v>
-      </c>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="b">
-        <v>0</v>
-      </c>
+      <c r="J83" t="n">
+        <v>-211.9</v>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="b">
+        <v>0</v>
+      </c>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="b">
+        <v>0</v>
+      </c>
+      <c r="O83" t="inlineStr"/>
       <c r="P83" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4785,19 +5037,22 @@
       <c r="I84" t="n">
         <v>34.25</v>
       </c>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="b">
-        <v>0</v>
-      </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="b">
-        <v>0</v>
-      </c>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="b">
-        <v>0</v>
-      </c>
+      <c r="J84" t="n">
+        <v>-207.84</v>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="b">
+        <v>0</v>
+      </c>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="b">
+        <v>0</v>
+      </c>
+      <c r="O84" t="inlineStr"/>
       <c r="P84" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q84" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4835,19 +5090,22 @@
       <c r="I85" t="n">
         <v>34.38</v>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="b">
-        <v>0</v>
-      </c>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="b">
-        <v>0</v>
-      </c>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="b">
-        <v>0</v>
-      </c>
+      <c r="J85" t="n">
+        <v>-206.71</v>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="b">
+        <v>0</v>
+      </c>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="b">
+        <v>0</v>
+      </c>
+      <c r="O85" t="inlineStr"/>
       <c r="P85" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4885,19 +5143,22 @@
       <c r="I86" t="n">
         <v>32.63</v>
       </c>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="b">
-        <v>0</v>
-      </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="b">
-        <v>0</v>
-      </c>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="b">
-        <v>0</v>
-      </c>
+      <c r="J86" t="n">
+        <v>-218.4</v>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="b">
+        <v>0</v>
+      </c>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="b">
+        <v>0</v>
+      </c>
+      <c r="O86" t="inlineStr"/>
       <c r="P86" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q86" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4935,19 +5196,22 @@
       <c r="I87" t="n">
         <v>35.35</v>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="b">
-        <v>0</v>
-      </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="b">
-        <v>0</v>
-      </c>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="b">
-        <v>0</v>
-      </c>
+      <c r="J87" t="n">
+        <v>-201.05</v>
+      </c>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="b">
+        <v>0</v>
+      </c>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="b">
+        <v>0</v>
+      </c>
+      <c r="O87" t="inlineStr"/>
       <c r="P87" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q87" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4985,19 +5249,22 @@
       <c r="I88" t="n">
         <v>36.11</v>
       </c>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="b">
-        <v>0</v>
-      </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="b">
-        <v>0</v>
-      </c>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="b">
-        <v>0</v>
-      </c>
+      <c r="J88" t="n">
+        <v>-196.1</v>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="b">
+        <v>0</v>
+      </c>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="b">
+        <v>0</v>
+      </c>
+      <c r="O88" t="inlineStr"/>
       <c r="P88" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q88" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5035,19 +5302,22 @@
       <c r="I89" t="n">
         <v>34.56</v>
       </c>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="b">
-        <v>0</v>
-      </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="b">
-        <v>0</v>
-      </c>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="b">
-        <v>0</v>
-      </c>
+      <c r="J89" t="n">
+        <v>-208.04</v>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="b">
+        <v>0</v>
+      </c>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="b">
+        <v>0</v>
+      </c>
+      <c r="O89" t="inlineStr"/>
       <c r="P89" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q89" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5085,19 +5355,22 @@
       <c r="I90" t="n">
         <v>34.91</v>
       </c>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="b">
-        <v>0</v>
-      </c>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="b">
-        <v>0</v>
-      </c>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="b">
-        <v>0</v>
-      </c>
+      <c r="J90" t="n">
+        <v>-205.43</v>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="b">
+        <v>0</v>
+      </c>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="b">
+        <v>0</v>
+      </c>
+      <c r="O90" t="inlineStr"/>
       <c r="P90" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q90" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5135,19 +5408,22 @@
       <c r="I91" t="n">
         <v>34.86</v>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="b">
-        <v>0</v>
-      </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="b">
-        <v>0</v>
-      </c>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="b">
-        <v>0</v>
-      </c>
+      <c r="J91" t="n">
+        <v>-204.71</v>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="b">
+        <v>0</v>
+      </c>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="b">
+        <v>0</v>
+      </c>
+      <c r="O91" t="inlineStr"/>
       <c r="P91" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5185,19 +5461,22 @@
       <c r="I92" t="n">
         <v>31.31</v>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="b">
-        <v>0</v>
-      </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="b">
-        <v>0</v>
-      </c>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="b">
-        <v>0</v>
-      </c>
+      <c r="J92" t="n">
+        <v>-227.18</v>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="b">
+        <v>0</v>
+      </c>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="b">
+        <v>0</v>
+      </c>
+      <c r="O92" t="inlineStr"/>
       <c r="P92" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5235,19 +5514,22 @@
       <c r="I93" t="n">
         <v>34.44</v>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="b">
-        <v>0</v>
-      </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="b">
-        <v>0</v>
-      </c>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="b">
-        <v>0</v>
-      </c>
+      <c r="J93" t="n">
+        <v>-205.98</v>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="b">
+        <v>0</v>
+      </c>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="b">
+        <v>0</v>
+      </c>
+      <c r="O93" t="inlineStr"/>
       <c r="P93" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5285,19 +5567,22 @@
       <c r="I94" t="n">
         <v>35.47</v>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="b">
-        <v>0</v>
-      </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="b">
-        <v>0</v>
-      </c>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="b">
-        <v>0</v>
-      </c>
+      <c r="J94" t="n">
+        <v>-201</v>
+      </c>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="b">
+        <v>0</v>
+      </c>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="b">
+        <v>0</v>
+      </c>
+      <c r="O94" t="inlineStr"/>
       <c r="P94" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q94" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5335,19 +5620,22 @@
       <c r="I95" t="n">
         <v>34.99</v>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="b">
-        <v>0</v>
-      </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="b">
-        <v>0</v>
-      </c>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="b">
-        <v>0</v>
-      </c>
+      <c r="J95" t="n">
+        <v>-207.5</v>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="b">
+        <v>0</v>
+      </c>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="b">
+        <v>0</v>
+      </c>
+      <c r="O95" t="inlineStr"/>
       <c r="P95" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q95" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5385,19 +5673,22 @@
       <c r="I96" t="n">
         <v>35.07</v>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="b">
-        <v>0</v>
-      </c>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="b">
-        <v>0</v>
-      </c>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="b">
-        <v>0</v>
-      </c>
+      <c r="J96" t="n">
+        <v>-202.94</v>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="b">
+        <v>0</v>
+      </c>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="b">
+        <v>0</v>
+      </c>
+      <c r="O96" t="inlineStr"/>
       <c r="P96" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q96" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5435,19 +5726,22 @@
       <c r="I97" t="n">
         <v>29.68</v>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="b">
-        <v>0</v>
-      </c>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="b">
-        <v>0</v>
-      </c>
-      <c r="N97" t="inlineStr"/>
-      <c r="O97" t="b">
-        <v>0</v>
-      </c>
+      <c r="J97" t="n">
+        <v>-244.24</v>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="b">
+        <v>0</v>
+      </c>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="b">
+        <v>0</v>
+      </c>
+      <c r="O97" t="inlineStr"/>
       <c r="P97" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5485,19 +5779,22 @@
       <c r="I98" t="n">
         <v>34.88</v>
       </c>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="b">
-        <v>0</v>
-      </c>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="b">
-        <v>0</v>
-      </c>
-      <c r="N98" t="inlineStr"/>
-      <c r="O98" t="b">
-        <v>0</v>
-      </c>
+      <c r="J98" t="n">
+        <v>-205.23</v>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="b">
+        <v>0</v>
+      </c>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="b">
+        <v>0</v>
+      </c>
+      <c r="O98" t="inlineStr"/>
       <c r="P98" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q98" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5535,19 +5832,22 @@
       <c r="I99" t="n">
         <v>34.51</v>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="b">
-        <v>0</v>
-      </c>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="b">
-        <v>0</v>
-      </c>
-      <c r="N99" t="inlineStr"/>
-      <c r="O99" t="b">
-        <v>0</v>
-      </c>
+      <c r="J99" t="n">
+        <v>-209.72</v>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="b">
+        <v>0</v>
+      </c>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="b">
+        <v>0</v>
+      </c>
+      <c r="O99" t="inlineStr"/>
       <c r="P99" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest results (2026-05-19_20-25-41)
</commit_message>
<xml_diff>
--- a/res/csv/data_by_date.xlsx
+++ b/res/csv/data_by_date.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q99"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -449,13 +449,14 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,35 +512,40 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>vpi_status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>reason_ER_dB</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_ER_dB</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>reason_IL_dB</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_IL_dB</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>reason_Vpi_V</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>out_of_bound_Vpi_V</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>is_problematic</t>
         </is>
@@ -582,19 +588,24 @@
       <c r="J2" t="n">
         <v>-180.3</v>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -635,19 +646,24 @@
       <c r="J3" t="n">
         <v>-166.8</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="b">
-        <v>0</v>
-      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -688,19 +704,24 @@
       <c r="J4" t="n">
         <v>-166.41</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="b">
-        <v>0</v>
-      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -741,19 +762,24 @@
       <c r="J5" t="n">
         <v>-186.65</v>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -794,19 +820,24 @@
       <c r="J6" t="n">
         <v>-172.51</v>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -847,19 +878,24 @@
       <c r="J7" t="n">
         <v>-161.57</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="b">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="b">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -900,19 +936,24 @@
       <c r="J8" t="n">
         <v>-186.21</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="b">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="b">
+        <v>0</v>
+      </c>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -953,19 +994,24 @@
       <c r="J9" t="n">
         <v>-179.2</v>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="b">
-        <v>0</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="b">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1006,19 +1052,24 @@
       <c r="J10" t="n">
         <v>-162.44</v>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="b">
-        <v>0</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="b">
-        <v>0</v>
-      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="b">
+        <v>0</v>
+      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1059,19 +1110,24 @@
       <c r="J11" t="n">
         <v>-178.67</v>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="b">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1112,19 +1168,24 @@
       <c r="J12" t="n">
         <v>-173.13</v>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="b">
-        <v>0</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="b">
-        <v>0</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="b">
-        <v>0</v>
-      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="b">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="b">
+        <v>0</v>
+      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1165,19 +1226,24 @@
       <c r="J13" t="n">
         <v>-177.9</v>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="b">
-        <v>0</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="b">
-        <v>0</v>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="b">
-        <v>0</v>
-      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="b">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="b">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1218,19 +1284,24 @@
       <c r="J14" t="n">
         <v>-178.79</v>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="b">
-        <v>0</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="b">
-        <v>0</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="b">
-        <v>0</v>
-      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="b">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="b">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="b">
+        <v>0</v>
+      </c>
+      <c r="R14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1271,19 +1342,24 @@
       <c r="J15" t="n">
         <v>-169.78</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="b">
-        <v>0</v>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="b">
-        <v>0</v>
-      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="b">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1324,23 +1400,28 @@
       <c r="J16" t="n">
         <v>3.13</v>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="b">
-        <v>0</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=3.13 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P16" t="b">
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="b">
+        <v>0</v>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=3.13)</t>
+        </is>
+      </c>
+      <c r="Q16" t="b">
         <v>1</v>
       </c>
-      <c r="Q16" s="2" t="b">
+      <c r="R16" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1381,23 +1462,28 @@
       <c r="J17" t="n">
         <v>2.3</v>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="b">
-        <v>0</v>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=2.30 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P17" t="b">
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="b">
+        <v>0</v>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=2.30)</t>
+        </is>
+      </c>
+      <c r="Q17" t="b">
         <v>1</v>
       </c>
-      <c r="Q17" s="2" t="b">
+      <c r="R17" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1438,23 +1524,28 @@
       <c r="J18" t="n">
         <v>-0.06</v>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="b">
-        <v>0</v>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="b">
-        <v>0</v>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.06 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P18" t="b">
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="b">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="b">
+        <v>0</v>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.06)</t>
+        </is>
+      </c>
+      <c r="Q18" t="b">
         <v>1</v>
       </c>
-      <c r="Q18" s="2" t="b">
+      <c r="R18" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1495,23 +1586,28 @@
       <c r="J19" t="n">
         <v>0.59</v>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="b">
-        <v>0</v>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="b">
-        <v>0</v>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.59 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P19" t="b">
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="b">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="b">
+        <v>0</v>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.59)</t>
+        </is>
+      </c>
+      <c r="Q19" t="b">
         <v>1</v>
       </c>
-      <c r="Q19" s="2" t="b">
+      <c r="R19" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1552,23 +1648,28 @@
       <c r="J20" t="n">
         <v>0.15</v>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="b">
-        <v>0</v>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="b">
-        <v>0</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.15 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P20" t="b">
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="b">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="b">
+        <v>0</v>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.15)</t>
+        </is>
+      </c>
+      <c r="Q20" t="b">
         <v>1</v>
       </c>
-      <c r="Q20" s="2" t="b">
+      <c r="R20" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1609,23 +1710,28 @@
       <c r="J21" t="n">
         <v>1.16</v>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="b">
-        <v>0</v>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="b">
-        <v>0</v>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.16 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P21" t="b">
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="b">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="b">
+        <v>0</v>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.16)</t>
+        </is>
+      </c>
+      <c r="Q21" t="b">
         <v>1</v>
       </c>
-      <c r="Q21" s="2" t="b">
+      <c r="R21" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1666,23 +1772,28 @@
       <c r="J22" t="n">
         <v>-4.66</v>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="b">
-        <v>0</v>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="b">
-        <v>0</v>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=4.66 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P22" t="b">
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="b">
+        <v>0</v>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=4.66)</t>
+        </is>
+      </c>
+      <c r="Q22" t="b">
         <v>1</v>
       </c>
-      <c r="Q22" s="2" t="b">
+      <c r="R22" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1723,23 +1834,28 @@
       <c r="J23" t="n">
         <v>-1.61</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="b">
-        <v>0</v>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="b">
-        <v>0</v>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.61 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P23" t="b">
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="b">
+        <v>0</v>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.61)</t>
+        </is>
+      </c>
+      <c r="Q23" t="b">
         <v>1</v>
       </c>
-      <c r="Q23" s="2" t="b">
+      <c r="R23" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1780,23 +1896,28 @@
       <c r="J24" t="n">
         <v>0.21</v>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="b">
-        <v>0</v>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="b">
-        <v>0</v>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.21 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P24" t="b">
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="b">
+        <v>0</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="b">
+        <v>0</v>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.21)</t>
+        </is>
+      </c>
+      <c r="Q24" t="b">
         <v>1</v>
       </c>
-      <c r="Q24" s="2" t="b">
+      <c r="R24" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1837,23 +1958,28 @@
       <c r="J25" t="n">
         <v>-1.2</v>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="b">
-        <v>0</v>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="b">
-        <v>0</v>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.20 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P25" t="b">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="b">
+        <v>0</v>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.20)</t>
+        </is>
+      </c>
+      <c r="Q25" t="b">
         <v>1</v>
       </c>
-      <c r="Q25" s="2" t="b">
+      <c r="R25" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1894,23 +2020,28 @@
       <c r="J26" t="n">
         <v>1.35</v>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="b">
-        <v>0</v>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="b">
-        <v>0</v>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.35 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P26" t="b">
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="b">
+        <v>0</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.35)</t>
+        </is>
+      </c>
+      <c r="Q26" t="b">
         <v>1</v>
       </c>
-      <c r="Q26" s="2" t="b">
+      <c r="R26" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1951,23 +2082,28 @@
       <c r="J27" t="n">
         <v>2.31</v>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="b">
-        <v>0</v>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="b">
-        <v>0</v>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=2.31 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P27" t="b">
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="b">
+        <v>0</v>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="b">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=2.31)</t>
+        </is>
+      </c>
+      <c r="Q27" t="b">
         <v>1</v>
       </c>
-      <c r="Q27" s="2" t="b">
+      <c r="R27" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2008,23 +2144,28 @@
       <c r="J28" t="n">
         <v>-0.08</v>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="b">
-        <v>0</v>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="b">
-        <v>0</v>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.08 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P28" t="b">
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="b">
+        <v>0</v>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="b">
+        <v>0</v>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.08)</t>
+        </is>
+      </c>
+      <c r="Q28" t="b">
         <v>1</v>
       </c>
-      <c r="Q28" s="2" t="b">
+      <c r="R28" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2065,23 +2206,28 @@
       <c r="J29" t="n">
         <v>1.3</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="b">
-        <v>0</v>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="b">
-        <v>0</v>
-      </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.30 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P29" t="b">
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="b">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="b">
+        <v>0</v>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.30)</t>
+        </is>
+      </c>
+      <c r="Q29" t="b">
         <v>1</v>
       </c>
-      <c r="Q29" s="2" t="b">
+      <c r="R29" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2122,23 +2268,28 @@
       <c r="J30" t="n">
         <v>0.91</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="b">
-        <v>0</v>
-      </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="b">
-        <v>0</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.91 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P30" t="b">
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="b">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="b">
+        <v>0</v>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.91)</t>
+        </is>
+      </c>
+      <c r="Q30" t="b">
         <v>1</v>
       </c>
-      <c r="Q30" s="2" t="b">
+      <c r="R30" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2179,23 +2330,28 @@
       <c r="J31" t="n">
         <v>0.28</v>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="b">
-        <v>0</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="b">
-        <v>0</v>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.28 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P31" t="b">
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="b">
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="b">
+        <v>0</v>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.28)</t>
+        </is>
+      </c>
+      <c r="Q31" t="b">
         <v>1</v>
       </c>
-      <c r="Q31" s="2" t="b">
+      <c r="R31" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2236,23 +2392,28 @@
       <c r="J32" t="n">
         <v>0.27</v>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="b">
-        <v>0</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="b">
-        <v>0</v>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.27 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P32" t="b">
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="b">
+        <v>0</v>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.27)</t>
+        </is>
+      </c>
+      <c r="Q32" t="b">
         <v>1</v>
       </c>
-      <c r="Q32" s="2" t="b">
+      <c r="R32" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2293,23 +2454,28 @@
       <c r="J33" t="n">
         <v>1.33</v>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="b">
-        <v>0</v>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="b">
-        <v>0</v>
-      </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.33 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P33" t="b">
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="b">
+        <v>0</v>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.33)</t>
+        </is>
+      </c>
+      <c r="Q33" t="b">
         <v>1</v>
       </c>
-      <c r="Q33" s="2" t="b">
+      <c r="R33" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2350,23 +2516,28 @@
       <c r="J34" t="n">
         <v>0.61</v>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="b">
-        <v>0</v>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="b">
-        <v>0</v>
-      </c>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.61 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P34" t="b">
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="b">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="b">
+        <v>0</v>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.61)</t>
+        </is>
+      </c>
+      <c r="Q34" t="b">
         <v>1</v>
       </c>
-      <c r="Q34" s="2" t="b">
+      <c r="R34" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2407,23 +2578,28 @@
       <c r="J35" t="n">
         <v>0.3</v>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="b">
-        <v>0</v>
-      </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="b">
-        <v>0</v>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.30 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P35" t="b">
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="b">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="b">
+        <v>0</v>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.30)</t>
+        </is>
+      </c>
+      <c r="Q35" t="b">
         <v>1</v>
       </c>
-      <c r="Q35" s="2" t="b">
+      <c r="R35" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2464,23 +2640,28 @@
       <c r="J36" t="n">
         <v>1.76</v>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="b">
-        <v>0</v>
-      </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="b">
-        <v>0</v>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.76 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P36" t="b">
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="b">
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="b">
+        <v>0</v>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.76)</t>
+        </is>
+      </c>
+      <c r="Q36" t="b">
         <v>1</v>
       </c>
-      <c r="Q36" s="2" t="b">
+      <c r="R36" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2521,23 +2702,28 @@
       <c r="J37" t="n">
         <v>-1.84</v>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="b">
-        <v>0</v>
-      </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="b">
-        <v>0</v>
-      </c>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=1.84 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P37" t="b">
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="b">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="b">
+        <v>0</v>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=1.84)</t>
+        </is>
+      </c>
+      <c r="Q37" t="b">
         <v>1</v>
       </c>
-      <c r="Q37" s="2" t="b">
+      <c r="R37" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2578,23 +2764,28 @@
       <c r="J38" t="n">
         <v>-0.57</v>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="b">
-        <v>0</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="b">
-        <v>0</v>
-      </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.57 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P38" t="b">
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="b">
+        <v>0</v>
+      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="b">
+        <v>0</v>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.57)</t>
+        </is>
+      </c>
+      <c r="Q38" t="b">
         <v>1</v>
       </c>
-      <c r="Q38" s="2" t="b">
+      <c r="R38" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2635,23 +2826,28 @@
       <c r="J39" t="n">
         <v>0.11</v>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="b">
-        <v>0</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="b">
-        <v>0</v>
-      </c>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.11 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P39" t="b">
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="b">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="b">
+        <v>0</v>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.11)</t>
+        </is>
+      </c>
+      <c r="Q39" t="b">
         <v>1</v>
       </c>
-      <c r="Q39" s="2" t="b">
+      <c r="R39" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2692,23 +2888,28 @@
       <c r="J40" t="n">
         <v>3.44</v>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="b">
-        <v>0</v>
-      </c>
-      <c r="O40" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=3.44 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P40" t="b">
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="b">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="b">
+        <v>0</v>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=3.44)</t>
+        </is>
+      </c>
+      <c r="Q40" t="b">
         <v>1</v>
       </c>
-      <c r="Q40" s="2" t="b">
+      <c r="R40" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2749,23 +2950,28 @@
       <c r="J41" t="n">
         <v>0.87</v>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="b">
-        <v>0</v>
-      </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="b">
-        <v>0</v>
-      </c>
-      <c r="O41" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.87 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P41" t="b">
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="b">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="b">
+        <v>0</v>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.87)</t>
+        </is>
+      </c>
+      <c r="Q41" t="b">
         <v>1</v>
       </c>
-      <c r="Q41" s="2" t="b">
+      <c r="R41" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2806,23 +3012,28 @@
       <c r="J42" t="n">
         <v>-0.88</v>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="b">
-        <v>0</v>
-      </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="b">
-        <v>0</v>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.88 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P42" t="b">
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="b">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="b">
+        <v>0</v>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.88)</t>
+        </is>
+      </c>
+      <c r="Q42" t="b">
         <v>1</v>
       </c>
-      <c r="Q42" s="2" t="b">
+      <c r="R42" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2863,23 +3074,28 @@
       <c r="J43" t="n">
         <v>-0.71</v>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="b">
-        <v>0</v>
-      </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="b">
-        <v>0</v>
-      </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>broken: |dλ/dV|=0.71 &lt; 10 pm/V (slope filter)</t>
-        </is>
-      </c>
-      <c r="P43" t="b">
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>slope_filter</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="b">
+        <v>0</v>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="b">
+        <v>0</v>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>broken: |dλ/dV| &lt; 10 pm/V (slope filter, |dλ/dV|=0.71)</t>
+        </is>
+      </c>
+      <c r="Q43" t="b">
         <v>1</v>
       </c>
-      <c r="Q43" s="2" t="b">
+      <c r="R43" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2920,19 +3136,24 @@
       <c r="J44" t="n">
         <v>-133.85</v>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="b">
-        <v>0</v>
-      </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="b">
-        <v>0</v>
-      </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="b">
-        <v>0</v>
-      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="b">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="b">
+        <v>0</v>
+      </c>
+      <c r="P44" t="inlineStr"/>
       <c r="Q44" t="b">
+        <v>0</v>
+      </c>
+      <c r="R44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2973,19 +3194,24 @@
       <c r="J45" t="n">
         <v>-116.09</v>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="b">
-        <v>0</v>
-      </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="b">
-        <v>0</v>
-      </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="b">
-        <v>0</v>
-      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="b">
+        <v>0</v>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="b">
+        <v>0</v>
+      </c>
+      <c r="P45" t="inlineStr"/>
       <c r="Q45" t="b">
+        <v>0</v>
+      </c>
+      <c r="R45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3026,19 +3252,24 @@
       <c r="J46" t="n">
         <v>-116.4</v>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="b">
-        <v>0</v>
-      </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="b">
-        <v>0</v>
-      </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="b">
-        <v>0</v>
-      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="b">
+        <v>0</v>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="b">
+        <v>0</v>
+      </c>
+      <c r="P46" t="inlineStr"/>
       <c r="Q46" t="b">
+        <v>0</v>
+      </c>
+      <c r="R46" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3079,19 +3310,24 @@
       <c r="J47" t="n">
         <v>-137.06</v>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="b">
-        <v>0</v>
-      </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="b">
-        <v>0</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="b">
-        <v>0</v>
-      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="b">
+        <v>0</v>
+      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="b">
+        <v>0</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="b">
+        <v>0</v>
+      </c>
+      <c r="R47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3132,19 +3368,24 @@
       <c r="J48" t="n">
         <v>-107.06</v>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="b">
-        <v>0</v>
-      </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="b">
-        <v>0</v>
-      </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="b">
-        <v>0</v>
-      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="b">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P48" t="inlineStr"/>
       <c r="Q48" t="b">
+        <v>0</v>
+      </c>
+      <c r="R48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3185,19 +3426,24 @@
       <c r="J49" t="n">
         <v>-112.21</v>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="b">
-        <v>0</v>
-      </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="b">
-        <v>0</v>
-      </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="b">
-        <v>0</v>
-      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="b">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="b">
+        <v>0</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
       <c r="Q49" t="b">
+        <v>0</v>
+      </c>
+      <c r="R49" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3238,19 +3484,24 @@
       <c r="J50" t="n">
         <v>-140.86</v>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="b">
-        <v>0</v>
-      </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="b">
-        <v>0</v>
-      </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="b">
-        <v>0</v>
-      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="b">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="b">
+        <v>0</v>
+      </c>
+      <c r="P50" t="inlineStr"/>
       <c r="Q50" t="b">
+        <v>0</v>
+      </c>
+      <c r="R50" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3291,19 +3542,24 @@
       <c r="J51" t="n">
         <v>-128.09</v>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="b">
-        <v>0</v>
-      </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="b">
-        <v>0</v>
-      </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="b">
-        <v>0</v>
-      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="b">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="b">
+        <v>0</v>
+      </c>
+      <c r="P51" t="inlineStr"/>
       <c r="Q51" t="b">
+        <v>0</v>
+      </c>
+      <c r="R51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3344,19 +3600,24 @@
       <c r="J52" t="n">
         <v>-106.92</v>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="b">
-        <v>0</v>
-      </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="b">
-        <v>0</v>
-      </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="b">
-        <v>0</v>
-      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="b">
+        <v>0</v>
+      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="b">
+        <v>0</v>
+      </c>
+      <c r="P52" t="inlineStr"/>
       <c r="Q52" t="b">
+        <v>0</v>
+      </c>
+      <c r="R52" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3397,19 +3658,24 @@
       <c r="J53" t="n">
         <v>-120.67</v>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="b">
-        <v>0</v>
-      </c>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="b">
-        <v>0</v>
-      </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="b">
-        <v>0</v>
-      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="b">
+        <v>0</v>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="b">
+        <v>0</v>
+      </c>
+      <c r="P53" t="inlineStr"/>
       <c r="Q53" t="b">
+        <v>0</v>
+      </c>
+      <c r="R53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3450,19 +3716,24 @@
       <c r="J54" t="n">
         <v>-130.6</v>
       </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="b">
-        <v>0</v>
-      </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="b">
-        <v>0</v>
-      </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="b">
-        <v>0</v>
-      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="b">
+        <v>0</v>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="b">
+        <v>0</v>
+      </c>
+      <c r="P54" t="inlineStr"/>
       <c r="Q54" t="b">
+        <v>0</v>
+      </c>
+      <c r="R54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3503,19 +3774,24 @@
       <c r="J55" t="n">
         <v>-118.08</v>
       </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="b">
-        <v>0</v>
-      </c>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="b">
-        <v>0</v>
-      </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="b">
-        <v>0</v>
-      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="b">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="b">
+        <v>0</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
       <c r="Q55" t="b">
+        <v>0</v>
+      </c>
+      <c r="R55" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3556,19 +3832,24 @@
       <c r="J56" t="n">
         <v>-115.51</v>
       </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="b">
-        <v>0</v>
-      </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="b">
-        <v>0</v>
-      </c>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="b">
-        <v>0</v>
-      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="b">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="b">
+        <v>0</v>
+      </c>
+      <c r="P56" t="inlineStr"/>
       <c r="Q56" t="b">
+        <v>0</v>
+      </c>
+      <c r="R56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3609,19 +3890,24 @@
       <c r="J57" t="n">
         <v>-129.17</v>
       </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="b">
-        <v>0</v>
-      </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="b">
-        <v>0</v>
-      </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="b">
-        <v>0</v>
-      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="b">
+        <v>0</v>
+      </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="b">
+        <v>0</v>
+      </c>
+      <c r="P57" t="inlineStr"/>
       <c r="Q57" t="b">
+        <v>0</v>
+      </c>
+      <c r="R57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3662,19 +3948,24 @@
       <c r="J58" t="n">
         <v>-118.03</v>
       </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="b">
-        <v>0</v>
-      </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="b">
-        <v>0</v>
-      </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="b">
-        <v>0</v>
-      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="b">
+        <v>0</v>
+      </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="b">
+        <v>0</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
       <c r="Q58" t="b">
+        <v>0</v>
+      </c>
+      <c r="R58" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3715,19 +4006,24 @@
       <c r="J59" t="n">
         <v>-130.75</v>
       </c>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="b">
-        <v>0</v>
-      </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="b">
-        <v>0</v>
-      </c>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="b">
-        <v>0</v>
-      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="b">
+        <v>0</v>
+      </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="b">
+        <v>0</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
       <c r="Q59" t="b">
+        <v>0</v>
+      </c>
+      <c r="R59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3768,19 +4064,24 @@
       <c r="J60" t="n">
         <v>-127.31</v>
       </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="b">
-        <v>0</v>
-      </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="b">
-        <v>0</v>
-      </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="b">
-        <v>0</v>
-      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="b">
+        <v>0</v>
+      </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="b">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
       <c r="Q60" t="b">
+        <v>0</v>
+      </c>
+      <c r="R60" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3821,19 +4122,24 @@
       <c r="J61" t="n">
         <v>-121.69</v>
       </c>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="b">
-        <v>0</v>
-      </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="b">
-        <v>0</v>
-      </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="b">
-        <v>0</v>
-      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="b">
+        <v>0</v>
+      </c>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="b">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
       <c r="Q61" t="b">
+        <v>0</v>
+      </c>
+      <c r="R61" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3874,19 +4180,24 @@
       <c r="J62" t="n">
         <v>-123.84</v>
       </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="b">
-        <v>0</v>
-      </c>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="b">
-        <v>0</v>
-      </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="b">
-        <v>0</v>
-      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="b">
+        <v>0</v>
+      </c>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="b">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr"/>
       <c r="Q62" t="b">
+        <v>0</v>
+      </c>
+      <c r="R62" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3927,19 +4238,24 @@
       <c r="J63" t="n">
         <v>-111.39</v>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="b">
-        <v>0</v>
-      </c>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="b">
-        <v>0</v>
-      </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="b">
-        <v>0</v>
-      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="b">
+        <v>0</v>
+      </c>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="b">
+        <v>0</v>
+      </c>
+      <c r="P63" t="inlineStr"/>
       <c r="Q63" t="b">
+        <v>0</v>
+      </c>
+      <c r="R63" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3980,19 +4296,24 @@
       <c r="J64" t="n">
         <v>-128.72</v>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="b">
-        <v>0</v>
-      </c>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="b">
-        <v>0</v>
-      </c>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="b">
-        <v>0</v>
-      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="b">
+        <v>0</v>
+      </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="b">
+        <v>0</v>
+      </c>
+      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="b">
+        <v>0</v>
+      </c>
+      <c r="R64" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4033,19 +4354,24 @@
       <c r="J65" t="n">
         <v>-113.59</v>
       </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="b">
-        <v>0</v>
-      </c>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="b">
-        <v>0</v>
-      </c>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="b">
-        <v>0</v>
-      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="b">
+        <v>0</v>
+      </c>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="b">
+        <v>0</v>
+      </c>
+      <c r="P65" t="inlineStr"/>
       <c r="Q65" t="b">
+        <v>0</v>
+      </c>
+      <c r="R65" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4086,19 +4412,24 @@
       <c r="J66" t="n">
         <v>-114.23</v>
       </c>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="b">
-        <v>0</v>
-      </c>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="b">
-        <v>0</v>
-      </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="b">
-        <v>0</v>
-      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="b">
+        <v>0</v>
+      </c>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="b">
+        <v>0</v>
+      </c>
+      <c r="P66" t="inlineStr"/>
       <c r="Q66" t="b">
+        <v>0</v>
+      </c>
+      <c r="R66" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4139,19 +4470,24 @@
       <c r="J67" t="n">
         <v>-117.58</v>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="b">
-        <v>0</v>
-      </c>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="b">
-        <v>0</v>
-      </c>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="b">
-        <v>0</v>
-      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="b">
+        <v>0</v>
+      </c>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="b">
+        <v>0</v>
+      </c>
+      <c r="P67" t="inlineStr"/>
       <c r="Q67" t="b">
+        <v>0</v>
+      </c>
+      <c r="R67" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4192,19 +4528,24 @@
       <c r="J68" t="n">
         <v>-121.84</v>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="b">
-        <v>0</v>
-      </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="b">
-        <v>0</v>
-      </c>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="b">
-        <v>0</v>
-      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="b">
+        <v>0</v>
+      </c>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="b">
+        <v>0</v>
+      </c>
+      <c r="P68" t="inlineStr"/>
       <c r="Q68" t="b">
+        <v>0</v>
+      </c>
+      <c r="R68" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4245,19 +4586,24 @@
       <c r="J69" t="n">
         <v>-107.66</v>
       </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="b">
-        <v>0</v>
-      </c>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="b">
-        <v>0</v>
-      </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="b">
-        <v>0</v>
-      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="b">
+        <v>0</v>
+      </c>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="b">
+        <v>0</v>
+      </c>
+      <c r="P69" t="inlineStr"/>
       <c r="Q69" t="b">
+        <v>0</v>
+      </c>
+      <c r="R69" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4298,19 +4644,24 @@
       <c r="J70" t="n">
         <v>-112.15</v>
       </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="b">
-        <v>0</v>
-      </c>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="b">
-        <v>0</v>
-      </c>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="b">
-        <v>0</v>
-      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="b">
+        <v>0</v>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="b">
+        <v>0</v>
+      </c>
+      <c r="P70" t="inlineStr"/>
       <c r="Q70" t="b">
+        <v>0</v>
+      </c>
+      <c r="R70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4351,19 +4702,24 @@
       <c r="J71" t="n">
         <v>-123.04</v>
       </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="b">
-        <v>0</v>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="b">
-        <v>0</v>
-      </c>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="b">
-        <v>0</v>
-      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="b">
+        <v>0</v>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="b">
+        <v>0</v>
+      </c>
+      <c r="P71" t="inlineStr"/>
       <c r="Q71" t="b">
+        <v>0</v>
+      </c>
+      <c r="R71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4404,19 +4760,24 @@
       <c r="J72" t="n">
         <v>-220.01</v>
       </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="b">
-        <v>0</v>
-      </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="b">
-        <v>0</v>
-      </c>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="b">
-        <v>0</v>
-      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="b">
+        <v>0</v>
+      </c>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="b">
+        <v>0</v>
+      </c>
+      <c r="P72" t="inlineStr"/>
       <c r="Q72" t="b">
+        <v>0</v>
+      </c>
+      <c r="R72" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4457,19 +4818,24 @@
       <c r="J73" t="n">
         <v>-218.92</v>
       </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="b">
-        <v>0</v>
-      </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="b">
-        <v>0</v>
-      </c>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="b">
-        <v>0</v>
-      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="b">
+        <v>0</v>
+      </c>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="b">
+        <v>0</v>
+      </c>
+      <c r="P73" t="inlineStr"/>
       <c r="Q73" t="b">
+        <v>0</v>
+      </c>
+      <c r="R73" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4510,19 +4876,24 @@
       <c r="J74" t="n">
         <v>-208.32</v>
       </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="b">
-        <v>0</v>
-      </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="b">
-        <v>0</v>
-      </c>
-      <c r="O74" t="inlineStr"/>
-      <c r="P74" t="b">
-        <v>0</v>
-      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="b">
+        <v>0</v>
+      </c>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="b">
+        <v>0</v>
+      </c>
+      <c r="P74" t="inlineStr"/>
       <c r="Q74" t="b">
+        <v>0</v>
+      </c>
+      <c r="R74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4563,19 +4934,24 @@
       <c r="J75" t="n">
         <v>-222.17</v>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="b">
-        <v>0</v>
-      </c>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="b">
-        <v>0</v>
-      </c>
-      <c r="O75" t="inlineStr"/>
-      <c r="P75" t="b">
-        <v>0</v>
-      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="b">
+        <v>0</v>
+      </c>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="b">
+        <v>0</v>
+      </c>
+      <c r="P75" t="inlineStr"/>
       <c r="Q75" t="b">
+        <v>0</v>
+      </c>
+      <c r="R75" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4616,19 +4992,24 @@
       <c r="J76" t="n">
         <v>-224.07</v>
       </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="b">
-        <v>0</v>
-      </c>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="b">
-        <v>0</v>
-      </c>
-      <c r="O76" t="inlineStr"/>
-      <c r="P76" t="b">
-        <v>0</v>
-      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="b">
+        <v>0</v>
+      </c>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="b">
+        <v>0</v>
+      </c>
+      <c r="P76" t="inlineStr"/>
       <c r="Q76" t="b">
+        <v>0</v>
+      </c>
+      <c r="R76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4669,19 +5050,24 @@
       <c r="J77" t="n">
         <v>-191.68</v>
       </c>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="b">
-        <v>0</v>
-      </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="b">
-        <v>0</v>
-      </c>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="b">
-        <v>0</v>
-      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="b">
+        <v>0</v>
+      </c>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="b">
+        <v>0</v>
+      </c>
+      <c r="P77" t="inlineStr"/>
       <c r="Q77" t="b">
+        <v>0</v>
+      </c>
+      <c r="R77" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4722,19 +5108,24 @@
       <c r="J78" t="n">
         <v>-202.41</v>
       </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="b">
-        <v>0</v>
-      </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="b">
-        <v>0</v>
-      </c>
-      <c r="O78" t="inlineStr"/>
-      <c r="P78" t="b">
-        <v>0</v>
-      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="b">
+        <v>0</v>
+      </c>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="b">
+        <v>0</v>
+      </c>
+      <c r="P78" t="inlineStr"/>
       <c r="Q78" t="b">
+        <v>0</v>
+      </c>
+      <c r="R78" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4775,19 +5166,24 @@
       <c r="J79" t="n">
         <v>-199.12</v>
       </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="b">
-        <v>0</v>
-      </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="b">
-        <v>0</v>
-      </c>
-      <c r="O79" t="inlineStr"/>
-      <c r="P79" t="b">
-        <v>0</v>
-      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="b">
+        <v>0</v>
+      </c>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="b">
+        <v>0</v>
+      </c>
+      <c r="P79" t="inlineStr"/>
       <c r="Q79" t="b">
+        <v>0</v>
+      </c>
+      <c r="R79" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4828,19 +5224,24 @@
       <c r="J80" t="n">
         <v>-214.56</v>
       </c>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="b">
-        <v>0</v>
-      </c>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="b">
-        <v>0</v>
-      </c>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="b">
-        <v>0</v>
-      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="b">
+        <v>0</v>
+      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="b">
+        <v>0</v>
+      </c>
+      <c r="P80" t="inlineStr"/>
       <c r="Q80" t="b">
+        <v>0</v>
+      </c>
+      <c r="R80" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4881,19 +5282,24 @@
       <c r="J81" t="n">
         <v>-204.04</v>
       </c>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="b">
-        <v>0</v>
-      </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="b">
-        <v>0</v>
-      </c>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="b">
-        <v>0</v>
-      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="b">
+        <v>0</v>
+      </c>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="b">
+        <v>0</v>
+      </c>
+      <c r="P81" t="inlineStr"/>
       <c r="Q81" t="b">
+        <v>0</v>
+      </c>
+      <c r="R81" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4934,19 +5340,24 @@
       <c r="J82" t="n">
         <v>-203.22</v>
       </c>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="b">
-        <v>0</v>
-      </c>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="b">
-        <v>0</v>
-      </c>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="b">
-        <v>0</v>
-      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="b">
+        <v>0</v>
+      </c>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="b">
+        <v>0</v>
+      </c>
+      <c r="P82" t="inlineStr"/>
       <c r="Q82" t="b">
+        <v>0</v>
+      </c>
+      <c r="R82" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4987,19 +5398,24 @@
       <c r="J83" t="n">
         <v>-211.9</v>
       </c>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="b">
-        <v>0</v>
-      </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="b">
-        <v>0</v>
-      </c>
-      <c r="O83" t="inlineStr"/>
-      <c r="P83" t="b">
-        <v>0</v>
-      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="b">
+        <v>0</v>
+      </c>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="b">
+        <v>0</v>
+      </c>
+      <c r="P83" t="inlineStr"/>
       <c r="Q83" t="b">
+        <v>0</v>
+      </c>
+      <c r="R83" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5040,19 +5456,24 @@
       <c r="J84" t="n">
         <v>-207.84</v>
       </c>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="b">
-        <v>0</v>
-      </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="b">
-        <v>0</v>
-      </c>
-      <c r="O84" t="inlineStr"/>
-      <c r="P84" t="b">
-        <v>0</v>
-      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="b">
+        <v>0</v>
+      </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="b">
+        <v>0</v>
+      </c>
+      <c r="P84" t="inlineStr"/>
       <c r="Q84" t="b">
+        <v>0</v>
+      </c>
+      <c r="R84" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5093,19 +5514,24 @@
       <c r="J85" t="n">
         <v>-206.71</v>
       </c>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="b">
-        <v>0</v>
-      </c>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="b">
-        <v>0</v>
-      </c>
-      <c r="O85" t="inlineStr"/>
-      <c r="P85" t="b">
-        <v>0</v>
-      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="b">
+        <v>0</v>
+      </c>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="b">
+        <v>0</v>
+      </c>
+      <c r="P85" t="inlineStr"/>
       <c r="Q85" t="b">
+        <v>0</v>
+      </c>
+      <c r="R85" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5146,19 +5572,24 @@
       <c r="J86" t="n">
         <v>-218.4</v>
       </c>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="b">
-        <v>0</v>
-      </c>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="b">
-        <v>0</v>
-      </c>
-      <c r="O86" t="inlineStr"/>
-      <c r="P86" t="b">
-        <v>0</v>
-      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="b">
+        <v>0</v>
+      </c>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="b">
+        <v>0</v>
+      </c>
+      <c r="P86" t="inlineStr"/>
       <c r="Q86" t="b">
+        <v>0</v>
+      </c>
+      <c r="R86" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5199,19 +5630,24 @@
       <c r="J87" t="n">
         <v>-201.05</v>
       </c>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="b">
-        <v>0</v>
-      </c>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="b">
-        <v>0</v>
-      </c>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="b">
-        <v>0</v>
-      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="b">
+        <v>0</v>
+      </c>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="b">
+        <v>0</v>
+      </c>
+      <c r="P87" t="inlineStr"/>
       <c r="Q87" t="b">
+        <v>0</v>
+      </c>
+      <c r="R87" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5252,19 +5688,24 @@
       <c r="J88" t="n">
         <v>-196.1</v>
       </c>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="b">
-        <v>0</v>
-      </c>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="b">
-        <v>0</v>
-      </c>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="b">
-        <v>0</v>
-      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="b">
+        <v>0</v>
+      </c>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="b">
+        <v>0</v>
+      </c>
+      <c r="P88" t="inlineStr"/>
       <c r="Q88" t="b">
+        <v>0</v>
+      </c>
+      <c r="R88" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5305,19 +5746,24 @@
       <c r="J89" t="n">
         <v>-208.04</v>
       </c>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="b">
-        <v>0</v>
-      </c>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="b">
-        <v>0</v>
-      </c>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="b">
-        <v>0</v>
-      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="b">
+        <v>0</v>
+      </c>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="b">
+        <v>0</v>
+      </c>
+      <c r="P89" t="inlineStr"/>
       <c r="Q89" t="b">
+        <v>0</v>
+      </c>
+      <c r="R89" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5358,19 +5804,24 @@
       <c r="J90" t="n">
         <v>-205.43</v>
       </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="b">
-        <v>0</v>
-      </c>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="b">
-        <v>0</v>
-      </c>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="b">
-        <v>0</v>
-      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="b">
+        <v>0</v>
+      </c>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="b">
+        <v>0</v>
+      </c>
+      <c r="P90" t="inlineStr"/>
       <c r="Q90" t="b">
+        <v>0</v>
+      </c>
+      <c r="R90" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5411,19 +5862,24 @@
       <c r="J91" t="n">
         <v>-204.71</v>
       </c>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="b">
-        <v>0</v>
-      </c>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="b">
-        <v>0</v>
-      </c>
-      <c r="O91" t="inlineStr"/>
-      <c r="P91" t="b">
-        <v>0</v>
-      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="b">
+        <v>0</v>
+      </c>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="b">
+        <v>0</v>
+      </c>
+      <c r="P91" t="inlineStr"/>
       <c r="Q91" t="b">
+        <v>0</v>
+      </c>
+      <c r="R91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5464,19 +5920,24 @@
       <c r="J92" t="n">
         <v>-227.18</v>
       </c>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="b">
-        <v>0</v>
-      </c>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="b">
-        <v>0</v>
-      </c>
-      <c r="O92" t="inlineStr"/>
-      <c r="P92" t="b">
-        <v>0</v>
-      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="b">
+        <v>0</v>
+      </c>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="b">
+        <v>0</v>
+      </c>
+      <c r="P92" t="inlineStr"/>
       <c r="Q92" t="b">
+        <v>0</v>
+      </c>
+      <c r="R92" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5517,19 +5978,24 @@
       <c r="J93" t="n">
         <v>-205.98</v>
       </c>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="b">
-        <v>0</v>
-      </c>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="b">
-        <v>0</v>
-      </c>
-      <c r="O93" t="inlineStr"/>
-      <c r="P93" t="b">
-        <v>0</v>
-      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="b">
+        <v>0</v>
+      </c>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="b">
+        <v>0</v>
+      </c>
+      <c r="P93" t="inlineStr"/>
       <c r="Q93" t="b">
+        <v>0</v>
+      </c>
+      <c r="R93" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5570,19 +6036,24 @@
       <c r="J94" t="n">
         <v>-201</v>
       </c>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="b">
-        <v>0</v>
-      </c>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="b">
-        <v>0</v>
-      </c>
-      <c r="O94" t="inlineStr"/>
-      <c r="P94" t="b">
-        <v>0</v>
-      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="b">
+        <v>0</v>
+      </c>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="b">
+        <v>0</v>
+      </c>
+      <c r="P94" t="inlineStr"/>
       <c r="Q94" t="b">
+        <v>0</v>
+      </c>
+      <c r="R94" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5623,19 +6094,24 @@
       <c r="J95" t="n">
         <v>-207.5</v>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="b">
-        <v>0</v>
-      </c>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="b">
-        <v>0</v>
-      </c>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="b">
-        <v>0</v>
-      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="b">
+        <v>0</v>
+      </c>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="b">
+        <v>0</v>
+      </c>
+      <c r="P95" t="inlineStr"/>
       <c r="Q95" t="b">
+        <v>0</v>
+      </c>
+      <c r="R95" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5676,19 +6152,24 @@
       <c r="J96" t="n">
         <v>-202.94</v>
       </c>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="b">
-        <v>0</v>
-      </c>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="b">
-        <v>0</v>
-      </c>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="b">
-        <v>0</v>
-      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="b">
+        <v>0</v>
+      </c>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="b">
+        <v>0</v>
+      </c>
+      <c r="P96" t="inlineStr"/>
       <c r="Q96" t="b">
+        <v>0</v>
+      </c>
+      <c r="R96" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5729,19 +6210,24 @@
       <c r="J97" t="n">
         <v>-244.24</v>
       </c>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="b">
-        <v>0</v>
-      </c>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="b">
-        <v>0</v>
-      </c>
-      <c r="O97" t="inlineStr"/>
-      <c r="P97" t="b">
-        <v>0</v>
-      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="b">
+        <v>0</v>
+      </c>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="b">
+        <v>0</v>
+      </c>
+      <c r="P97" t="inlineStr"/>
       <c r="Q97" t="b">
+        <v>0</v>
+      </c>
+      <c r="R97" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5782,19 +6268,24 @@
       <c r="J98" t="n">
         <v>-205.23</v>
       </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="b">
-        <v>0</v>
-      </c>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="b">
-        <v>0</v>
-      </c>
-      <c r="O98" t="inlineStr"/>
-      <c r="P98" t="b">
-        <v>0</v>
-      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="b">
+        <v>0</v>
+      </c>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="b">
+        <v>0</v>
+      </c>
+      <c r="P98" t="inlineStr"/>
       <c r="Q98" t="b">
+        <v>0</v>
+      </c>
+      <c r="R98" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5835,19 +6326,24 @@
       <c r="J99" t="n">
         <v>-209.72</v>
       </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="b">
-        <v>0</v>
-      </c>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="b">
-        <v>0</v>
-      </c>
-      <c r="O99" t="inlineStr"/>
-      <c r="P99" t="b">
-        <v>0</v>
-      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="b">
+        <v>0</v>
+      </c>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="b">
+        <v>0</v>
+      </c>
+      <c r="P99" t="inlineStr"/>
       <c r="Q99" t="b">
+        <v>0</v>
+      </c>
+      <c r="R99" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>